<commit_message>
Restructure budget to match LINGUA Africa Submittable form categories
Split coordinateurs from Personnel into a separate 'Data Collection &
Processing' line (14 × 100 × 8 = 11,200 USD), rename 'Équipement et
matériel' → 'Équipement et logiciels', renumber sections 3–7 → 4–8.
Personnel drops from 178,500 to 167,300 USD; total directs unchanged
at 209,500 USD; grand total cash unchanged at 220,000 USD.

Updated in: LINGUA_Africa_Application_QA.md, generate_application.py,
generate_application_en.py, generate_budget.py, and all three generated
artefacts (DOCX × 2, XLSX × 1).
</commit_message>
<xml_diff>
--- a/LINGUA_Africa_Budget_Detaille.xlsx
+++ b/LINGUA_Africa_Budget_Detaille.xlsx
@@ -895,11 +895,11 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>178500</v>
+        <v>167300</v>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>85.2 % des coûts directs</t>
+          <t>79.9 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       <c r="A10" s="1" t="inlineStr"/>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Équipement et matériel</t>
+          <t>Équipement et logiciels</t>
         </is>
       </c>
       <c r="C10" s="10" t="n">
@@ -915,7 +915,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>3.8 % des coûts directs</t>
+          <t xml:space="preserve"> 3.8 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -923,15 +923,15 @@
       <c r="A11" s="1" t="inlineStr"/>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Déplacements et terrain</t>
+          <t>Collecte et traitement de données</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>16000</v>
+        <v>11200</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>7.6 % des coûts directs</t>
+          <t xml:space="preserve"> 5.3 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -939,15 +939,15 @@
       <c r="A12" s="1" t="inlineStr"/>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Formation et ateliers</t>
+          <t>Déplacements et terrain</t>
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>4500</v>
+        <v>16000</v>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>2.1 % des coûts directs</t>
+          <t xml:space="preserve"> 7.6 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -955,15 +955,15 @@
       <c r="A13" s="1" t="inlineStr"/>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Communication et documentation</t>
+          <t>Formation et ateliers</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>1500</v>
+        <v>4500</v>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>0.7 % des coûts directs</t>
+          <t xml:space="preserve"> 2.1 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -971,112 +971,125 @@
       <c r="A14" s="1" t="inlineStr"/>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Autres coûts directs</t>
+          <t>Communication et documentation</t>
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>0.5 % des coûts directs</t>
+          <t xml:space="preserve"> 0.7 % des coûts directs</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="1" t="inlineStr"/>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Autres coûts directs</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 0.5 % des coûts directs</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="1" t="inlineStr"/>
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Sous-total coûts directs</t>
         </is>
       </c>
-      <c r="C15" s="13" t="n">
+      <c r="C16" s="13" t="n">
         <v>209500</v>
       </c>
-      <c r="D15" s="14" t="n"/>
-    </row>
-    <row r="16" ht="14" customHeight="1">
-      <c r="A16" s="1" t="inlineStr"/>
-    </row>
-    <row r="17" ht="28" customHeight="1">
+      <c r="D16" s="14" t="n"/>
+    </row>
+    <row r="17" ht="14" customHeight="1">
       <c r="A17" s="1" t="inlineStr"/>
-      <c r="B17" s="15" t="inlineStr">
-        <is>
-          <t>Frais généraux / indirects (5 %)</t>
-        </is>
-      </c>
-      <c r="C17" s="16" t="n">
-        <v>10500</v>
-      </c>
-      <c r="D17" s="17" t="inlineStr">
-        <is>
-          <t>5 % × 209 500</t>
-        </is>
-      </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="1" t="inlineStr"/>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>BUDGET CASH TOTAL DEMANDÉ</t>
-        </is>
-      </c>
-      <c r="C18" s="19" t="n">
-        <v>220000</v>
-      </c>
-      <c r="D18" s="20" t="inlineStr">
-        <is>
-          <t>&lt; 250 000 USD ✓</t>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Frais généraux / indirects (5 %)</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>10500</v>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>5 % × 209 500</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="1" t="inlineStr"/>
-      <c r="B19" s="21" t="inlineStr">
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>BUDGET CASH TOTAL DEMANDÉ</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="n">
+        <v>220000</v>
+      </c>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 250 000 USD ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="1" t="inlineStr"/>
+      <c r="B20" s="21" t="inlineStr">
         <is>
           <t>Crédits de calcul GCP (Q18)</t>
         </is>
       </c>
-      <c r="C19" s="22" t="n">
+      <c r="C20" s="22" t="n">
         <v>150000</v>
       </c>
-      <c r="D19" s="23" t="inlineStr">
+      <c r="D20" s="23" t="inlineStr">
         <is>
           <t>&lt; 400 000 USD ✓</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="14" customHeight="1">
-      <c r="A20" s="1" t="inlineStr"/>
-    </row>
-    <row r="21" ht="22" customHeight="1">
+    <row r="21" ht="14" customHeight="1">
       <c r="A21" s="1" t="inlineStr"/>
-      <c r="B21" s="24" t="inlineStr">
-        <is>
-          <t>Contact :</t>
-        </is>
-      </c>
-      <c r="C21" s="25" t="inlineStr">
-        <is>
-          <t>Fenitra Ravelomanantsoa — fenitra@google.com</t>
-        </is>
-      </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="1" t="inlineStr"/>
       <c r="B22" s="24" t="inlineStr">
         <is>
+          <t>Contact :</t>
+        </is>
+      </c>
+      <c r="C22" s="25" t="inlineStr">
+        <is>
+          <t>Fenitra Ravelomanantsoa — fenitra@google.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="1" t="inlineStr"/>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
           <t>Dépôt GitHub :</t>
         </is>
       </c>
-      <c r="C22" s="26" t="inlineStr">
+      <c r="C23" s="26" t="inlineStr">
         <is>
           <t>github.com/mgvaovao/ml  |  github.com/mgvaovao/backend_ia</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr"/>
@@ -1157,22 +1170,23 @@
       <c r="A49" s="1" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
     <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D16:E16"/>
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="D15:E15"/>
     <mergeCell ref="D19:E19"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="C23:E23"/>
     <mergeCell ref="C22:E22"/>
     <mergeCell ref="D14:E14"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="C7:E7"/>
-    <mergeCell ref="C21:E21"/>
     <mergeCell ref="D9:E9"/>
     <mergeCell ref="C6:E6"/>
   </mergeCells>
@@ -1186,7 +1200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1432,341 +1446,311 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="37" t="inlineStr">
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Personnel</t>
+        </is>
+      </c>
+      <c r="E12" s="44" t="n">
+        <v>167300</v>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>79.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>2. ÉQUIPEMENT ET LOGICIELS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="31" t="inlineStr">
+        <is>
+          <t>Ordinateurs portables — équipe technique locale (hors fondateur à Zurich)</t>
+        </is>
+      </c>
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>778 USD × 6 unités  (≈ 3 500 000 MGA l'unité)</t>
+        </is>
+      </c>
+      <c r="C14" s="33" t="inlineStr">
+        <is>
+          <t>unité</t>
+        </is>
+      </c>
+      <c r="D14" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" s="35" t="n">
+        <v>778</v>
+      </c>
+      <c r="F14" s="36" t="n">
+        <v>4667</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="37" t="inlineStr">
+        <is>
+          <t>Tablettes de terrain pour coordinateurs de collecte</t>
+        </is>
+      </c>
+      <c r="B15" s="38" t="inlineStr">
+        <is>
+          <t>150 × 14 coordinateurs</t>
+        </is>
+      </c>
+      <c r="C15" s="39" t="inlineStr">
+        <is>
+          <t>unité</t>
+        </is>
+      </c>
+      <c r="D15" s="40" t="n">
+        <v>14</v>
+      </c>
+      <c r="E15" s="41" t="n">
+        <v>150</v>
+      </c>
+      <c r="F15" s="42" t="n">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="31" t="inlineStr">
+        <is>
+          <t>Microphones USB qualité ASR/TTS pour les sessions de collecte</t>
+        </is>
+      </c>
+      <c r="B16" s="32" t="inlineStr">
+        <is>
+          <t>50 × 14 coordinateurs</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>unité</t>
+        </is>
+      </c>
+      <c r="D16" s="34" t="n">
+        <v>14</v>
+      </c>
+      <c r="E16" s="35" t="n">
+        <v>50</v>
+      </c>
+      <c r="F16" s="36" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="37" t="inlineStr">
+        <is>
+          <t>Matériel de connectivité (routeurs Wi-Fi, dongles 4G régions rurales)</t>
+        </is>
+      </c>
+      <c r="B17" s="38" t="inlineStr">
+        <is>
+          <t>Forfait — 14 régions à faible infrastructure</t>
+        </is>
+      </c>
+      <c r="C17" s="39" t="inlineStr">
+        <is>
+          <t>forfait</t>
+        </is>
+      </c>
+      <c r="D17" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="41" t="n">
+        <v>533</v>
+      </c>
+      <c r="F17" s="42" t="n">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Équipement et logiciels</t>
+        </is>
+      </c>
+      <c r="E18" s="44" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F18" s="17" t="inlineStr">
+        <is>
+          <t>3.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>3. COLLECTE ET TRAITEMENT DE DONNÉES</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>14 coordinateurs locaux de collecte terrain</t>
         </is>
       </c>
-      <c r="B12" s="38" t="inlineStr">
+      <c r="B20" s="32" t="inlineStr">
         <is>
           <t>100 × 14 pers. × 8 mois actifs</t>
         </is>
       </c>
-      <c r="C12" s="39" t="inlineStr">
+      <c r="C20" s="33" t="inlineStr">
         <is>
           <t>pers.×mois</t>
         </is>
       </c>
-      <c r="D12" s="40" t="n">
+      <c r="D20" s="34" t="n">
         <v>112</v>
       </c>
-      <c r="E12" s="41" t="n">
+      <c r="E20" s="35" t="n">
         <v>100</v>
       </c>
-      <c r="F12" s="42" t="n">
+      <c r="F20" s="36" t="n">
         <v>11200</v>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Personnel</t>
-        </is>
-      </c>
-      <c r="E13" s="44" t="n">
-        <v>178500</v>
-      </c>
-      <c r="F13" s="17" t="inlineStr">
-        <is>
-          <t>85.2%</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="30" t="inlineStr">
-        <is>
-          <t>2. ÉQUIPEMENT ET MATÉRIEL</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="31" t="inlineStr">
-        <is>
-          <t>Ordinateurs portables — équipe technique locale (hors fondateur à Zurich)</t>
-        </is>
-      </c>
-      <c r="B15" s="32" t="inlineStr">
-        <is>
-          <t>778 USD × 6 unités  (≈ 3 500 000 MGA l'unité)</t>
-        </is>
-      </c>
-      <c r="C15" s="33" t="inlineStr">
-        <is>
-          <t>unité</t>
-        </is>
-      </c>
-      <c r="D15" s="34" t="n">
-        <v>6</v>
-      </c>
-      <c r="E15" s="35" t="n">
-        <v>778</v>
-      </c>
-      <c r="F15" s="36" t="n">
-        <v>4667</v>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="37" t="inlineStr">
-        <is>
-          <t>Tablettes de terrain pour coordinateurs de collecte</t>
-        </is>
-      </c>
-      <c r="B16" s="38" t="inlineStr">
-        <is>
-          <t>150 × 14 coordinateurs</t>
-        </is>
-      </c>
-      <c r="C16" s="39" t="inlineStr">
-        <is>
-          <t>unité</t>
-        </is>
-      </c>
-      <c r="D16" s="40" t="n">
-        <v>14</v>
-      </c>
-      <c r="E16" s="41" t="n">
-        <v>150</v>
-      </c>
-      <c r="F16" s="42" t="n">
-        <v>2100</v>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="31" t="inlineStr">
-        <is>
-          <t>Microphones USB qualité ASR/TTS pour les sessions de collecte</t>
-        </is>
-      </c>
-      <c r="B17" s="32" t="inlineStr">
-        <is>
-          <t>50 × 14 coordinateurs</t>
-        </is>
-      </c>
-      <c r="C17" s="33" t="inlineStr">
-        <is>
-          <t>unité</t>
-        </is>
-      </c>
-      <c r="D17" s="34" t="n">
-        <v>14</v>
-      </c>
-      <c r="E17" s="35" t="n">
-        <v>50</v>
-      </c>
-      <c r="F17" s="36" t="n">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="37" t="inlineStr">
-        <is>
-          <t>Matériel de connectivité (routeurs Wi-Fi, dongles 4G régions rurales)</t>
-        </is>
-      </c>
-      <c r="B18" s="38" t="inlineStr">
-        <is>
-          <t>Forfait — 14 régions à faible infrastructure</t>
-        </is>
-      </c>
-      <c r="C18" s="39" t="inlineStr">
-        <is>
-          <t>forfait</t>
-        </is>
-      </c>
-      <c r="D18" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="41" t="n">
-        <v>533</v>
-      </c>
-      <c r="F18" s="42" t="n">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Équipement</t>
-        </is>
-      </c>
-      <c r="E19" s="44" t="n">
-        <v>8000</v>
-      </c>
-      <c r="F19" s="17" t="inlineStr">
-        <is>
-          <t>3.8%</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="30" t="inlineStr">
-        <is>
-          <t>3. DÉPLACEMENTS ET TERRAIN</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="31" t="inlineStr">
-        <is>
-          <t>Missions régionales — avions intérieurs + taxi-brousse (14 régions, 2 visites)</t>
-        </is>
-      </c>
-      <c r="B21" s="32" t="inlineStr">
-        <is>
-          <t>400 × 14 régions × 2 allers-retours</t>
-        </is>
-      </c>
-      <c r="C21" s="33" t="inlineStr">
-        <is>
-          <t>mission</t>
-        </is>
-      </c>
-      <c r="D21" s="34" t="n">
-        <v>28</v>
-      </c>
-      <c r="E21" s="35" t="n">
-        <v>400</v>
-      </c>
-      <c r="F21" s="36" t="n">
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Collecte et traitement de données</t>
+        </is>
+      </c>
+      <c r="E21" s="44" t="n">
         <v>11200</v>
       </c>
+      <c r="F21" s="17" t="inlineStr">
+        <is>
+          <t>5.3%</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="37" t="inlineStr">
-        <is>
-          <t>Per diem et hébergement — superviseurs terrain</t>
-        </is>
-      </c>
-      <c r="B22" s="38" t="inlineStr">
-        <is>
-          <t>50/j × 3 j × 14 régions × 2 visites</t>
-        </is>
-      </c>
-      <c r="C22" s="39" t="inlineStr">
-        <is>
-          <t>j×mission</t>
-        </is>
-      </c>
-      <c r="D22" s="40" t="n">
-        <v>84</v>
-      </c>
-      <c r="E22" s="41" t="n">
-        <v>50</v>
-      </c>
-      <c r="F22" s="42" t="n">
-        <v>4200</v>
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>4. DÉPLACEMENTS ET TERRAIN</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="31" t="inlineStr">
         <is>
-          <t>Location de salles communautaires pour les sessions de collecte</t>
+          <t>Missions régionales — avions intérieurs + taxi-brousse (14 régions, 2 visites)</t>
         </is>
       </c>
       <c r="B23" s="32" t="inlineStr">
         <is>
-          <t>43 × 14 régions × 2 sessions  +  réserve imprévus</t>
+          <t>400 × 14 régions × 2 allers-retours</t>
         </is>
       </c>
       <c r="C23" s="33" t="inlineStr">
         <is>
-          <t>session</t>
+          <t>mission</t>
         </is>
       </c>
       <c r="D23" s="34" t="n">
         <v>28</v>
       </c>
       <c r="E23" s="35" t="n">
+        <v>400</v>
+      </c>
+      <c r="F23" s="36" t="n">
+        <v>11200</v>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="37" t="inlineStr">
+        <is>
+          <t>Per diem et hébergement — superviseurs terrain</t>
+        </is>
+      </c>
+      <c r="B24" s="38" t="inlineStr">
+        <is>
+          <t>50/j × 3 j × 14 régions × 2 visites</t>
+        </is>
+      </c>
+      <c r="C24" s="39" t="inlineStr">
+        <is>
+          <t>j×mission</t>
+        </is>
+      </c>
+      <c r="D24" s="40" t="n">
+        <v>84</v>
+      </c>
+      <c r="E24" s="41" t="n">
+        <v>50</v>
+      </c>
+      <c r="F24" s="42" t="n">
+        <v>4200</v>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="31" t="inlineStr">
+        <is>
+          <t>Location de salles communautaires pour les sessions de collecte</t>
+        </is>
+      </c>
+      <c r="B25" s="32" t="inlineStr">
+        <is>
+          <t>43 × 14 régions × 2 sessions  +  réserve imprévus</t>
+        </is>
+      </c>
+      <c r="C25" s="33" t="inlineStr">
+        <is>
+          <t>session</t>
+        </is>
+      </c>
+      <c r="D25" s="34" t="n">
+        <v>28</v>
+      </c>
+      <c r="E25" s="35" t="n">
         <v>43</v>
       </c>
-      <c r="F23" s="36" t="n">
+      <c r="F25" s="36" t="n">
         <v>600</v>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="43" t="inlineStr">
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="43" t="inlineStr">
         <is>
           <t>Sous-total Déplacements &amp; terrain</t>
         </is>
       </c>
-      <c r="E24" s="44" t="n">
+      <c r="E26" s="44" t="n">
         <v>16000</v>
       </c>
-      <c r="F24" s="17" t="inlineStr">
+      <c r="F26" s="17" t="inlineStr">
         <is>
           <t>7.6%</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="30" t="inlineStr">
-        <is>
-          <t>4. FORMATION ET ATELIERS</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="31" t="inlineStr">
-        <is>
-          <t>Formation des 14 coordinateurs locaux (protocoles, outils d'enregistrement)</t>
-        </is>
-      </c>
-      <c r="B26" s="32" t="inlineStr">
-        <is>
-          <t>Salle + matériel + indemnités — 2 jours</t>
-        </is>
-      </c>
-      <c r="C26" s="33" t="inlineStr">
-        <is>
-          <t>forfait</t>
-        </is>
-      </c>
-      <c r="D26" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="35" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F26" s="36" t="n">
-        <v>1500</v>
-      </c>
-    </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="37" t="inlineStr">
-        <is>
-          <t>Atelier de restitution final — communauté NLP africaine</t>
-        </is>
-      </c>
-      <c r="B27" s="38" t="inlineStr">
-        <is>
-          <t>Organisation, accueil participants, matériel de présentation</t>
-        </is>
-      </c>
-      <c r="C27" s="39" t="inlineStr">
-        <is>
-          <t>forfait</t>
-        </is>
-      </c>
-      <c r="D27" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="41" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F27" s="42" t="n">
-        <v>2000</v>
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>5. FORMATION ET ATELIERS</t>
+        </is>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="31" t="inlineStr">
         <is>
-          <t>Participation à une conférence NLP régionale (ex. IndabaX)</t>
+          <t>Formation des 14 coordinateurs locaux (protocoles, outils d'enregistrement)</t>
         </is>
       </c>
       <c r="B28" s="32" t="inlineStr">
         <is>
-          <t>Inscription + transport + hébergement</t>
+          <t>Salle + matériel + indemnités — 2 jours</t>
         </is>
       </c>
       <c r="C28" s="33" t="inlineStr">
@@ -1778,288 +1762,288 @@
         <v>1</v>
       </c>
       <c r="E28" s="35" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F28" s="36" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="37" t="inlineStr">
+        <is>
+          <t>Atelier de restitution final — communauté NLP africaine</t>
+        </is>
+      </c>
+      <c r="B29" s="38" t="inlineStr">
+        <is>
+          <t>Organisation, accueil participants, matériel de présentation</t>
+        </is>
+      </c>
+      <c r="C29" s="39" t="inlineStr">
+        <is>
+          <t>forfait</t>
+        </is>
+      </c>
+      <c r="D29" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="41" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F29" s="42" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="31" t="inlineStr">
+        <is>
+          <t>Participation à une conférence NLP régionale (ex. IndabaX)</t>
+        </is>
+      </c>
+      <c r="B30" s="32" t="inlineStr">
+        <is>
+          <t>Inscription + transport + hébergement</t>
+        </is>
+      </c>
+      <c r="C30" s="33" t="inlineStr">
+        <is>
+          <t>forfait</t>
+        </is>
+      </c>
+      <c r="D30" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="35" t="n">
         <v>1000</v>
       </c>
-      <c r="F28" s="36" t="n">
+      <c r="F30" s="36" t="n">
         <v>1000</v>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="43" t="inlineStr">
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="43" t="inlineStr">
         <is>
           <t>Sous-total Formation &amp; ateliers</t>
         </is>
       </c>
-      <c r="E29" s="44" t="n">
+      <c r="E31" s="44" t="n">
         <v>4500</v>
       </c>
-      <c r="F29" s="17" t="inlineStr">
+      <c r="F31" s="17" t="inlineStr">
         <is>
           <t>2.1%</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="30" t="inlineStr">
-        <is>
-          <t>5. COMMUNICATION ET DOCUMENTATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="31" t="inlineStr">
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>6. COMMUNICATION ET DOCUMENTATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="31" t="inlineStr">
         <is>
           <t>Rapports d'avancement semestriels (mise en page, traduction FR/EN)</t>
         </is>
       </c>
-      <c r="B31" s="32" t="inlineStr">
+      <c r="B33" s="32" t="inlineStr">
         <is>
           <t>250 × 6 rapports (M3, M6, M9, M12, M15, M18)</t>
         </is>
       </c>
-      <c r="C31" s="33" t="inlineStr">
+      <c r="C33" s="33" t="inlineStr">
         <is>
           <t>rapport</t>
         </is>
       </c>
-      <c r="D31" s="34" t="n">
+      <c r="D33" s="34" t="n">
         <v>6</v>
       </c>
-      <c r="E31" s="35" t="n">
+      <c r="E33" s="35" t="n">
         <v>100</v>
       </c>
-      <c r="F31" s="36" t="n">
+      <c r="F33" s="36" t="n">
         <v>600</v>
       </c>
     </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="37" t="inlineStr">
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="37" t="inlineStr">
         <is>
           <t>Outils numériques : gestion projet, hébergement web, licences</t>
         </is>
       </c>
-      <c r="B32" s="38" t="inlineStr">
+      <c r="B34" s="38" t="inlineStr">
         <is>
           <t>50/mois × 18 mois</t>
         </is>
       </c>
-      <c r="C32" s="39" t="inlineStr">
+      <c r="C34" s="39" t="inlineStr">
         <is>
           <t>mois</t>
         </is>
       </c>
-      <c r="D32" s="40" t="n">
+      <c r="D34" s="40" t="n">
         <v>18</v>
       </c>
-      <c r="E32" s="41" t="n">
+      <c r="E34" s="41" t="n">
         <v>50</v>
       </c>
-      <c r="F32" s="42" t="n">
+      <c r="F34" s="42" t="n">
         <v>900</v>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="43" t="inlineStr">
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="43" t="inlineStr">
         <is>
           <t>Sous-total Communication</t>
         </is>
       </c>
-      <c r="E33" s="44" t="n">
+      <c r="E35" s="44" t="n">
         <v>1500</v>
       </c>
-      <c r="F33" s="17" t="inlineStr">
+      <c r="F35" s="17" t="inlineStr">
         <is>
           <t>0.7%</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="30" t="inlineStr">
-        <is>
-          <t>6. AUTRES COÛTS DIRECTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="31" t="inlineStr">
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="30" t="inlineStr">
+        <is>
+          <t>7. AUTRES COÛTS DIRECTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="31" t="inlineStr">
         <is>
           <t>Frais administratifs et juridiques (contrats, enregistrements officiels)</t>
         </is>
       </c>
-      <c r="B35" s="32" t="inlineStr">
+      <c r="B37" s="32" t="inlineStr">
         <is>
           <t>Notaire, administration, légalisation</t>
         </is>
       </c>
-      <c r="C35" s="33" t="inlineStr">
+      <c r="C37" s="33" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D35" s="34" t="n">
+      <c r="D37" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="E35" s="35" t="n">
+      <c r="E37" s="35" t="n">
         <v>500</v>
       </c>
-      <c r="F35" s="36" t="n">
+      <c r="F37" s="36" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="37" t="inlineStr">
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="37" t="inlineStr">
         <is>
           <t>Réserve pour imprévus opérationnels</t>
         </is>
       </c>
-      <c r="B36" s="38" t="inlineStr">
+      <c r="B38" s="38" t="inlineStr">
         <is>
           <t>Ajustements terrain non anticipés</t>
         </is>
       </c>
-      <c r="C36" s="39" t="inlineStr">
+      <c r="C38" s="39" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D36" s="40" t="n">
+      <c r="D38" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E36" s="41" t="n">
+      <c r="E38" s="41" t="n">
         <v>500</v>
       </c>
-      <c r="F36" s="42" t="n">
+      <c r="F38" s="42" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="43" t="inlineStr">
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="43" t="inlineStr">
         <is>
           <t>Sous-total Autres coûts directs</t>
         </is>
       </c>
-      <c r="E37" s="44" t="n">
+      <c r="E39" s="44" t="n">
         <v>1000</v>
       </c>
-      <c r="F37" s="17" t="inlineStr">
+      <c r="F39" s="17" t="inlineStr">
         <is>
           <t>0.5%</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="45" t="inlineStr">
+    <row r="40" ht="24" customHeight="1">
+      <c r="A40" s="45" t="inlineStr">
         <is>
           <t>TOTAL DES COÛTS DIRECTS</t>
         </is>
       </c>
-      <c r="E38" s="46" t="n">
+      <c r="E40" s="46" t="n">
         <v>209500</v>
       </c>
-      <c r="F38" s="47" t="inlineStr">
+      <c r="F40" s="47" t="inlineStr">
         <is>
           <t>100 %</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="43" t="inlineStr">
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="43" t="inlineStr">
         <is>
           <t>Frais généraux / Coûts indirects (5 % des coûts directs)</t>
         </is>
       </c>
-      <c r="E39" s="44" t="n">
+      <c r="E41" s="44" t="n">
         <v>10500</v>
       </c>
-      <c r="F39" s="48" t="inlineStr">
+      <c r="F41" s="48" t="inlineStr">
         <is>
           <t>5 % × 209 500</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="28" customHeight="1">
-      <c r="A40" s="18" t="inlineStr">
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="18" t="inlineStr">
         <is>
           <t>GRAND TOTAL — BUDGET CASH DEMANDÉ  (plafond Cat. 3 : 250 000 USD)</t>
         </is>
       </c>
-      <c r="E40" s="49" t="n">
+      <c r="E42" s="49" t="n">
         <v>220000</v>
       </c>
-      <c r="F40" s="50" t="inlineStr">
+      <c r="F42" s="50" t="inlineStr">
         <is>
           <t>&lt; 250 000 USD ✓</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="51" t="inlineStr">
-        <is>
-          <t>7. RESSOURCES DE CALCUL GCP — Q18  (crédits séparés du budget cash — plafond 400 000 USD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="31" t="inlineStr">
-        <is>
-          <t>Vertex AI Custom Training — fine-tuning NLLB LoRA (6 langues × 18 dialectes)</t>
-        </is>
-      </c>
-      <c r="B43" s="32" t="inlineStr">
-        <is>
-          <t>L4 Spot ~0,28 $/h — expérimentations + runs finaux</t>
-        </is>
-      </c>
-      <c r="C43" s="33" t="inlineStr">
-        <is>
-          <t>forfait</t>
-        </is>
-      </c>
-      <c r="D43" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" s="35" t="n">
-        <v>45000</v>
-      </c>
-      <c r="F43" s="36" t="n">
-        <v>45000</v>
-      </c>
-    </row>
     <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="37" t="inlineStr">
-        <is>
-          <t>Vertex AI Custom Training — fine-tuning MMS-TTS VITS (18 dialectes)</t>
-        </is>
-      </c>
-      <c r="B44" s="38" t="inlineStr">
-        <is>
-          <t>18 dialectes × 3 cycles × 1,5 h GPU + hyperparamètres</t>
-        </is>
-      </c>
-      <c r="C44" s="39" t="inlineStr">
-        <is>
-          <t>forfait</t>
-        </is>
-      </c>
-      <c r="D44" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" s="41" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F44" s="42" t="n">
-        <v>20000</v>
+      <c r="A44" s="51" t="inlineStr">
+        <is>
+          <t>8. RESSOURCES DE CALCUL GCP — Q18  (crédits séparés du budget cash — plafond 400 000 USD)</t>
+        </is>
       </c>
     </row>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="31" t="inlineStr">
         <is>
-          <t>Vertex AI Custom Training — buffer expérimentation &amp; réentraînement</t>
+          <t>Vertex AI Custom Training — fine-tuning NLLB LoRA (6 langues × 18 dialectes)</t>
         </is>
       </c>
       <c r="B45" s="32" t="inlineStr">
         <is>
-          <t>Nouvelles données M10–M18, réentraînements itératifs</t>
+          <t>L4 Spot ~0,28 $/h — expérimentations + runs finaux</t>
         </is>
       </c>
       <c r="C45" s="33" t="inlineStr">
@@ -2071,47 +2055,47 @@
         <v>1</v>
       </c>
       <c r="E45" s="35" t="n">
-        <v>15000</v>
+        <v>45000</v>
       </c>
       <c r="F45" s="36" t="n">
-        <v>15000</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="37" t="inlineStr">
         <is>
-          <t>Cloud Run GPU (NVIDIA L4 24 Go) — API MGVaovao en production</t>
+          <t>Vertex AI Custom Training — fine-tuning MMS-TTS VITS (18 dialectes)</t>
         </is>
       </c>
       <c r="B46" s="38" t="inlineStr">
         <is>
-          <t>~2 500 $/mois × 18 mois — scale-to-zero hors heures</t>
+          <t>18 dialectes × 3 cycles × 1,5 h GPU + hyperparamètres</t>
         </is>
       </c>
       <c r="C46" s="39" t="inlineStr">
         <is>
-          <t>mois</t>
+          <t>forfait</t>
         </is>
       </c>
       <c r="D46" s="40" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E46" s="41" t="n">
-        <v>2500</v>
+        <v>20000</v>
       </c>
       <c r="F46" s="42" t="n">
-        <v>45000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="31" t="inlineStr">
         <is>
-          <t>GCS — stockage corpus audio + checkpoints (≈ 3 To)</t>
+          <t>Vertex AI Custom Training — buffer expérimentation &amp; réentraînement</t>
         </is>
       </c>
       <c r="B47" s="32" t="inlineStr">
         <is>
-          <t>0,02 $/Go/mois × 3 000 Go × 18 mois + egress</t>
+          <t>Nouvelles données M10–M18, réentraînements itératifs</t>
         </is>
       </c>
       <c r="C47" s="33" t="inlineStr">
@@ -2123,73 +2107,73 @@
         <v>1</v>
       </c>
       <c r="E47" s="35" t="n">
-        <v>1500</v>
+        <v>15000</v>
       </c>
       <c r="F47" s="36" t="n">
-        <v>1500</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="37" t="inlineStr">
         <is>
-          <t>Vertex AI Pipelines — orchestration MLOps Kubeflow DAG</t>
+          <t>Cloud Run GPU (NVIDIA L4 24 Go) — API MGVaovao en production</t>
         </is>
       </c>
       <c r="B48" s="38" t="inlineStr">
         <is>
-          <t>0,03 $/run × ~500 runs + monitoring continu</t>
+          <t>~2 500 $/mois × 18 mois — scale-to-zero hors heures</t>
         </is>
       </c>
       <c r="C48" s="39" t="inlineStr">
         <is>
-          <t>forfait</t>
+          <t>mois</t>
         </is>
       </c>
       <c r="D48" s="40" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="E48" s="41" t="n">
-        <v>500</v>
+        <v>2500</v>
       </c>
       <c r="F48" s="42" t="n">
-        <v>500</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="31" t="inlineStr">
         <is>
-          <t>Cloud Build, Artifact Registry, Cloud Monitoring, Pub/Sub</t>
+          <t>GCS — stockage corpus audio + checkpoints (≈ 3 To)</t>
         </is>
       </c>
       <c r="B49" s="32" t="inlineStr">
         <is>
-          <t>CI/CD, registre d'images, alertes, déclencheurs GCS</t>
+          <t>0,02 $/Go/mois × 3 000 Go × 18 mois + egress</t>
         </is>
       </c>
       <c r="C49" s="33" t="inlineStr">
         <is>
-          <t>mois</t>
+          <t>forfait</t>
         </is>
       </c>
       <c r="D49" s="34" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E49" s="35" t="n">
-        <v>139</v>
+        <v>1500</v>
       </c>
       <c r="F49" s="36" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="37" t="inlineStr">
         <is>
-          <t>Dataflow / ingestion pipeline audio — traitement et normalisation</t>
+          <t>Vertex AI Pipelines — orchestration MLOps Kubeflow DAG</t>
         </is>
       </c>
       <c r="B50" s="38" t="inlineStr">
         <is>
-          <t>Ingestion et prétraitement audio en pipeline GCS</t>
+          <t>0,03 $/run × ~500 runs + monitoring continu</t>
         </is>
       </c>
       <c r="C50" s="39" t="inlineStr">
@@ -2201,48 +2185,102 @@
         <v>1</v>
       </c>
       <c r="E50" s="41" t="n">
+        <v>500</v>
+      </c>
+      <c r="F50" s="42" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="31" t="inlineStr">
+        <is>
+          <t>Cloud Build, Artifact Registry, Cloud Monitoring, Pub/Sub</t>
+        </is>
+      </c>
+      <c r="B51" s="32" t="inlineStr">
+        <is>
+          <t>CI/CD, registre d'images, alertes, déclencheurs GCS</t>
+        </is>
+      </c>
+      <c r="C51" s="33" t="inlineStr">
+        <is>
+          <t>mois</t>
+        </is>
+      </c>
+      <c r="D51" s="34" t="n">
+        <v>18</v>
+      </c>
+      <c r="E51" s="35" t="n">
+        <v>139</v>
+      </c>
+      <c r="F51" s="36" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="37" t="inlineStr">
+        <is>
+          <t>Dataflow / ingestion pipeline audio — traitement et normalisation</t>
+        </is>
+      </c>
+      <c r="B52" s="38" t="inlineStr">
+        <is>
+          <t>Ingestion et prétraitement audio en pipeline GCS</t>
+        </is>
+      </c>
+      <c r="C52" s="39" t="inlineStr">
+        <is>
+          <t>forfait</t>
+        </is>
+      </c>
+      <c r="D52" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="41" t="n">
         <v>20500</v>
       </c>
-      <c r="F50" s="42" t="n">
+      <c r="F52" s="42" t="n">
         <v>20500</v>
       </c>
     </row>
-    <row r="51" ht="28" customHeight="1">
-      <c r="A51" s="21" t="inlineStr">
+    <row r="53" ht="28" customHeight="1">
+      <c r="A53" s="21" t="inlineStr">
         <is>
           <t>TOTAL CRÉDITS GCP DEMANDÉS  (Q18b — séparé du budget cash)</t>
         </is>
       </c>
-      <c r="E51" s="52" t="n">
+      <c r="E53" s="52" t="n">
         <v>150000</v>
       </c>
-      <c r="F51" s="53" t="inlineStr">
+      <c r="F53" s="53" t="inlineStr">
         <is>
           <t>&lt; 400 000 USD ✓</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A13:D13"/>
+  <mergeCells count="21">
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A27:F27"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A40:D40"/>
-    <mergeCell ref="A42:F42"/>
-    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A32:F32"/>
     <mergeCell ref="A39:D39"/>
-    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A42:D42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2254,7 +2292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2306,23 +2344,23 @@
         </is>
       </c>
       <c r="B4" s="58" t="n">
-        <v>178500</v>
+        <v>167300</v>
       </c>
       <c r="C4" s="59" t="inlineStr">
         <is>
-          <t>85.2 %</t>
+          <t>79.9 %</t>
         </is>
       </c>
       <c r="D4" s="59" t="inlineStr">
         <is>
-          <t>Équipe complète 18 mois — 8 postes + 14 coordinateurs</t>
+          <t>Équipe permanente 18 mois — 7 postes</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="60" t="inlineStr">
         <is>
-          <t>2. Équipement et matériel</t>
+          <t>2. Équipement et logiciels</t>
         </is>
       </c>
       <c r="B5" s="61" t="n">
@@ -2342,225 +2380,245 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="57" t="inlineStr">
         <is>
-          <t>3. Déplacements et terrain</t>
+          <t>3. Collecte et traitement de données</t>
         </is>
       </c>
       <c r="B6" s="58" t="n">
-        <v>16000</v>
+        <v>11200</v>
       </c>
       <c r="C6" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 7.6 %</t>
+          <t xml:space="preserve"> 5.3 %</t>
         </is>
       </c>
       <c r="D6" s="59" t="inlineStr">
         <is>
-          <t>14 régions × 2 missions — avion + taxi-brousse</t>
+          <t>14 coordinateurs locaux terrain × 8 mois × 100 USD</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="60" t="inlineStr">
         <is>
-          <t>4. Formation et ateliers</t>
+          <t>4. Déplacements et terrain</t>
         </is>
       </c>
       <c r="B7" s="61" t="n">
-        <v>4500</v>
+        <v>16000</v>
       </c>
       <c r="C7" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 2.1 %</t>
+          <t xml:space="preserve"> 7.6 %</t>
         </is>
       </c>
       <c r="D7" s="62" t="inlineStr">
         <is>
-          <t>Formation coordinateurs + atelier restitution + conférence</t>
+          <t>14 régions × 2 missions — avion + taxi-brousse</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="57" t="inlineStr">
         <is>
-          <t>5. Communication et documentation</t>
+          <t>5. Formation et ateliers</t>
         </is>
       </c>
       <c r="B8" s="58" t="n">
-        <v>1500</v>
+        <v>4500</v>
       </c>
       <c r="C8" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 0.7 %</t>
+          <t xml:space="preserve"> 2.1 %</t>
         </is>
       </c>
       <c r="D8" s="59" t="inlineStr">
         <is>
-          <t>Rapports, outils numériques</t>
+          <t>Formation coordinateurs + atelier restitution + conférence</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="60" t="inlineStr">
         <is>
-          <t>6. Autres coûts directs</t>
+          <t>6. Communication et documentation</t>
         </is>
       </c>
       <c r="B9" s="61" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C9" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 0.7 %</t>
+        </is>
+      </c>
+      <c r="D9" s="62" t="inlineStr">
+        <is>
+          <t>Rapports, outils numériques</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="57" t="inlineStr">
+        <is>
+          <t>7. Autres coûts directs</t>
+        </is>
+      </c>
+      <c r="B10" s="58" t="n">
         <v>1000</v>
       </c>
-      <c r="C9" s="62" t="inlineStr">
+      <c r="C10" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve"> 0.5 %</t>
         </is>
       </c>
-      <c r="D9" s="62" t="inlineStr">
+      <c r="D10" s="59" t="inlineStr">
         <is>
           <t>Frais administratifs + réserve imprévus</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="63" t="inlineStr">
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="63" t="inlineStr">
         <is>
           <t>TOTAL DES COÛTS DIRECTS</t>
         </is>
       </c>
-      <c r="B10" s="46" t="n">
+      <c r="B11" s="46" t="n">
         <v>209500</v>
       </c>
-      <c r="C10" s="47" t="inlineStr">
+      <c r="C11" s="47" t="inlineStr">
         <is>
           <t>100 %</t>
         </is>
       </c>
-      <c r="D10" s="47" t="inlineStr">
+      <c r="D11" s="47" t="inlineStr">
         <is>
           <t>209 500 USD</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="64" t="inlineStr">
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="64" t="inlineStr">
         <is>
           <t>Frais généraux / indirects (5 %)</t>
         </is>
       </c>
-      <c r="B11" s="44" t="n">
+      <c r="B12" s="44" t="n">
         <v>10500</v>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>5 %</t>
         </is>
       </c>
-      <c r="D11" s="17" t="inlineStr">
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>5 % × 209 500</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="65" t="inlineStr">
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="65" t="inlineStr">
         <is>
           <t>GRAND TOTAL — BUDGET CASH DEMANDÉ</t>
         </is>
       </c>
-      <c r="B12" s="49" t="n">
+      <c r="B13" s="49" t="n">
         <v>220000</v>
       </c>
-      <c r="C12" s="66" t="inlineStr">
+      <c r="C13" s="66" t="inlineStr">
         <is>
           <t>&lt; 250 000 USD ✓</t>
         </is>
       </c>
-      <c r="D12" s="66" t="inlineStr">
+      <c r="D13" s="66" t="inlineStr">
         <is>
           <t>Plafond Cat. 3 respecté</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="67" t="inlineStr">
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="67" t="inlineStr">
         <is>
           <t>RESSOURCES DE CALCUL GCP — Q18  (séparées du budget cash — plafond 400 000 USD)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="57" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="57" t="inlineStr">
         <is>
           <t>Vertex AI Custom Training — NLLB LoRA + MMS-TTS + expérimentation</t>
         </is>
       </c>
-      <c r="B15" s="58" t="n">
+      <c r="B16" s="58" t="n">
         <v>80000</v>
       </c>
-      <c r="C15" s="59" t="inlineStr">
+      <c r="C16" s="59" t="inlineStr">
         <is>
           <t>53.3 %</t>
         </is>
       </c>
-      <c r="D15" s="59" t="inlineStr">
+      <c r="D16" s="59" t="inlineStr">
         <is>
           <t>6 langues × 18 dialectes + cycles itératifs</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="60" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="60" t="inlineStr">
         <is>
           <t>Cloud Run GPU — infrastructure de production API (18 mois)</t>
         </is>
       </c>
-      <c r="B16" s="61" t="n">
+      <c r="B17" s="61" t="n">
         <v>45000</v>
       </c>
-      <c r="C16" s="62" t="inlineStr">
+      <c r="C17" s="62" t="inlineStr">
         <is>
           <t>30.0 %</t>
         </is>
       </c>
-      <c r="D16" s="62" t="inlineStr">
+      <c r="D17" s="62" t="inlineStr">
         <is>
           <t>NVIDIA L4 24 Go — scale-to-zero hors heures</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="57" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="57" t="inlineStr">
         <is>
           <t>GCS, Pipelines, CI/CD, Monitoring, Dataflow, Pub/Sub</t>
         </is>
       </c>
-      <c r="B17" s="58" t="n">
+      <c r="B18" s="58" t="n">
         <v>25000</v>
       </c>
-      <c r="C17" s="59" t="inlineStr">
+      <c r="C18" s="59" t="inlineStr">
         <is>
           <t>16.7 %</t>
         </is>
       </c>
-      <c r="D17" s="59" t="inlineStr">
+      <c r="D18" s="59" t="inlineStr">
         <is>
           <t>Stockage 3 To + orchestration MLOps + ingestion</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="68" t="inlineStr">
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="68" t="inlineStr">
         <is>
           <t>TOTAL CRÉDITS GCP DEMANDÉS (Q18b)</t>
         </is>
       </c>
-      <c r="B18" s="52" t="n">
+      <c r="B19" s="52" t="n">
         <v>150000</v>
       </c>
-      <c r="C18" s="69" t="inlineStr">
+      <c r="C19" s="69" t="inlineStr">
         <is>
           <t>&lt; 400 000 USD ✓</t>
         </is>
       </c>
-      <c r="D18" s="69" t="inlineStr">
+      <c r="D19" s="69" t="inlineStr">
         <is>
           <t>Plafond Q18 respecté</t>
         </is>
@@ -2569,8 +2627,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A14:D14"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A15:D15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Expand data team to 54 collectors + 36 annotators; devs as co-financing
- Separate collection (section 3) and annotation/ground truth (section 4)
  as distinct budget lines
- 54 field collectors (3/dialect × 18 dialects) at 600 000 MGA (133 USD)
  × 4 active months = 28 728 USD
- 36 annotators (2/dialect × 18 dialects) at 900 000 MGA (200 USD)
  × 4 active months = 28 800 USD
- Remove 2 junior AI devs from LINGUA Africa budget; all 8 developers
  (backend, frontend, IA, data science, DevOps) appear as organisation
  co-financing at 1 500 000 MGA/month × 18 months = 47 952 USD
- Personnel drops to 144 900 USD (core leadership only)
- New totals: directs 233 428 | overhead 11 671 | cash total 245 099 USD
  (still under the 250 000 USD Category 3 cap)
- Updated across: QA.md, generate_application.py, generate_application_en.py,
  generate_budget.py and all three generated artefacts
</commit_message>
<xml_diff>
--- a/LINGUA_Africa_Budget_Detaille.xlsx
+++ b/LINGUA_Africa_Budget_Detaille.xlsx
@@ -155,7 +155,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -195,6 +195,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F0F4F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -243,7 +248,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -373,13 +378,16 @@
     <xf numFmtId="3" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="15" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="15" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -427,7 +435,7 @@
     <xf numFmtId="0" fontId="22" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -891,15 +899,15 @@
       <c r="A9" s="1" t="inlineStr"/>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Personnel (salaires équipe)</t>
+          <t>Personnel — direction permanente</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>167300</v>
+        <v>144900</v>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>79.9 % des coûts directs</t>
+          <t>62.1 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -915,7 +923,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 3.8 % des coûts directs</t>
+          <t xml:space="preserve"> 3.4 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -923,15 +931,15 @@
       <c r="A11" s="1" t="inlineStr"/>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Collecte et traitement de données</t>
+          <t>Collecte terrain (54 collecteurs)</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>11200</v>
+        <v>28728</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 5.3 % des coûts directs</t>
+          <t>12.3 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -939,15 +947,15 @@
       <c r="A12" s="1" t="inlineStr"/>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Déplacements et terrain</t>
+          <t>Annotation ground truth (36 annotateurs)</t>
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>16000</v>
+        <v>28800</v>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 7.6 % des coûts directs</t>
+          <t>12.3 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -955,15 +963,15 @@
       <c r="A13" s="1" t="inlineStr"/>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Formation et ateliers</t>
+          <t>Déplacements et terrain</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>4500</v>
+        <v>16000</v>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 2.1 % des coûts directs</t>
+          <t xml:space="preserve"> 6.9 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -971,15 +979,15 @@
       <c r="A14" s="1" t="inlineStr"/>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Communication et documentation</t>
+          <t>Formation et ateliers</t>
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>1500</v>
+        <v>4500</v>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 0.7 % des coûts directs</t>
+          <t xml:space="preserve"> 1.9 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -987,15 +995,15 @@
       <c r="A15" s="1" t="inlineStr"/>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Autres coûts directs</t>
+          <t>Communication et autres coûts</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 0.5 % des coûts directs</t>
+          <t xml:space="preserve"> 1.1 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1015,7 @@
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>209500</v>
+        <v>233428</v>
       </c>
       <c r="D16" s="14" t="n"/>
     </row>
@@ -1022,11 +1030,11 @@
         </is>
       </c>
       <c r="C18" s="16" t="n">
-        <v>10500</v>
+        <v>11671</v>
       </c>
       <c r="D18" s="17" t="inlineStr">
         <is>
-          <t>5 % × 209 500</t>
+          <t>5 % × 233 428</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1046,7 @@
         </is>
       </c>
       <c r="C19" s="19" t="n">
-        <v>220000</v>
+        <v>245099</v>
       </c>
       <c r="D19" s="20" t="inlineStr">
         <is>
@@ -1200,7 +1208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1394,415 +1402,366 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="37" t="inlineStr">
-        <is>
-          <t>Développeur IA junior 1 (100 %)</t>
-        </is>
-      </c>
-      <c r="B10" s="38" t="inlineStr">
-        <is>
-          <t>800 × 18 mois</t>
-        </is>
-      </c>
-      <c r="C10" s="39" t="inlineStr">
-        <is>
-          <t>mois</t>
-        </is>
-      </c>
-      <c r="D10" s="40" t="n">
-        <v>18</v>
-      </c>
-      <c r="E10" s="41" t="n">
-        <v>800</v>
-      </c>
-      <c r="F10" s="42" t="n">
-        <v>14400</v>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="31" t="inlineStr">
-        <is>
-          <t>Développeur IA junior 2 (100 %, M9–M18)</t>
-        </is>
-      </c>
-      <c r="B11" s="32" t="inlineStr">
-        <is>
-          <t>800 × 10 mois</t>
-        </is>
-      </c>
-      <c r="C11" s="33" t="inlineStr">
-        <is>
-          <t>mois</t>
-        </is>
-      </c>
-      <c r="D11" s="34" t="n">
-        <v>10</v>
-      </c>
-      <c r="E11" s="35" t="n">
-        <v>800</v>
-      </c>
-      <c r="F11" s="36" t="n">
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Personnel (direction permanente)</t>
+        </is>
+      </c>
+      <c r="E10" s="44" t="n">
+        <v>144900</v>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>62.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="45" t="inlineStr">
+        <is>
+          <t>↳ Co-financement organisation (hors budget LINGUA Africa) : 8 développeurs (backend / frontend / IA / data science / DevOps) × 333 USD (1 500 000 MGA) × 18 mois = 47 952 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>2. ÉQUIPEMENT ET LOGICIELS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>Ordinateurs portables — équipe technique locale (hors fondateur à Zurich)</t>
+        </is>
+      </c>
+      <c r="B13" s="32" t="inlineStr">
+        <is>
+          <t>778 USD × 6 unités  (≈ 3 500 000 MGA l'unité)</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="inlineStr">
+        <is>
+          <t>unité</t>
+        </is>
+      </c>
+      <c r="D13" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" s="35" t="n">
+        <v>778</v>
+      </c>
+      <c r="F13" s="36" t="n">
+        <v>4667</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="37" t="inlineStr">
+        <is>
+          <t>Tablettes de terrain pour coordinateurs de collecte</t>
+        </is>
+      </c>
+      <c r="B14" s="38" t="inlineStr">
+        <is>
+          <t>150 × 14 coordinateurs</t>
+        </is>
+      </c>
+      <c r="C14" s="39" t="inlineStr">
+        <is>
+          <t>unité</t>
+        </is>
+      </c>
+      <c r="D14" s="40" t="n">
+        <v>14</v>
+      </c>
+      <c r="E14" s="41" t="n">
+        <v>150</v>
+      </c>
+      <c r="F14" s="42" t="n">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="31" t="inlineStr">
+        <is>
+          <t>Microphones USB qualité ASR/TTS pour les sessions de collecte</t>
+        </is>
+      </c>
+      <c r="B15" s="32" t="inlineStr">
+        <is>
+          <t>50 × 14 coordinateurs</t>
+        </is>
+      </c>
+      <c r="C15" s="33" t="inlineStr">
+        <is>
+          <t>unité</t>
+        </is>
+      </c>
+      <c r="D15" s="34" t="n">
+        <v>14</v>
+      </c>
+      <c r="E15" s="35" t="n">
+        <v>50</v>
+      </c>
+      <c r="F15" s="36" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="37" t="inlineStr">
+        <is>
+          <t>Matériel de connectivité (routeurs Wi-Fi, dongles 4G régions rurales)</t>
+        </is>
+      </c>
+      <c r="B16" s="38" t="inlineStr">
+        <is>
+          <t>Forfait — 14 régions à faible infrastructure</t>
+        </is>
+      </c>
+      <c r="C16" s="39" t="inlineStr">
+        <is>
+          <t>forfait</t>
+        </is>
+      </c>
+      <c r="D16" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="41" t="n">
+        <v>533</v>
+      </c>
+      <c r="F16" s="42" t="n">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Équipement et logiciels</t>
+        </is>
+      </c>
+      <c r="E17" s="44" t="n">
         <v>8000</v>
       </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Personnel</t>
-        </is>
-      </c>
-      <c r="E12" s="44" t="n">
-        <v>167300</v>
-      </c>
-      <c r="F12" s="17" t="inlineStr">
-        <is>
-          <t>79.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="30" t="inlineStr">
-        <is>
-          <t>2. ÉQUIPEMENT ET LOGICIELS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="31" t="inlineStr">
-        <is>
-          <t>Ordinateurs portables — équipe technique locale (hors fondateur à Zurich)</t>
-        </is>
-      </c>
-      <c r="B14" s="32" t="inlineStr">
-        <is>
-          <t>778 USD × 6 unités  (≈ 3 500 000 MGA l'unité)</t>
-        </is>
-      </c>
-      <c r="C14" s="33" t="inlineStr">
-        <is>
-          <t>unité</t>
-        </is>
-      </c>
-      <c r="D14" s="34" t="n">
-        <v>6</v>
-      </c>
-      <c r="E14" s="35" t="n">
-        <v>778</v>
-      </c>
-      <c r="F14" s="36" t="n">
-        <v>4667</v>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="37" t="inlineStr">
-        <is>
-          <t>Tablettes de terrain pour coordinateurs de collecte</t>
-        </is>
-      </c>
-      <c r="B15" s="38" t="inlineStr">
-        <is>
-          <t>150 × 14 coordinateurs</t>
-        </is>
-      </c>
-      <c r="C15" s="39" t="inlineStr">
-        <is>
-          <t>unité</t>
-        </is>
-      </c>
-      <c r="D15" s="40" t="n">
-        <v>14</v>
-      </c>
-      <c r="E15" s="41" t="n">
-        <v>150</v>
-      </c>
-      <c r="F15" s="42" t="n">
-        <v>2100</v>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="31" t="inlineStr">
-        <is>
-          <t>Microphones USB qualité ASR/TTS pour les sessions de collecte</t>
-        </is>
-      </c>
-      <c r="B16" s="32" t="inlineStr">
-        <is>
-          <t>50 × 14 coordinateurs</t>
-        </is>
-      </c>
-      <c r="C16" s="33" t="inlineStr">
-        <is>
-          <t>unité</t>
-        </is>
-      </c>
-      <c r="D16" s="34" t="n">
-        <v>14</v>
-      </c>
-      <c r="E16" s="35" t="n">
-        <v>50</v>
-      </c>
-      <c r="F16" s="36" t="n">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="37" t="inlineStr">
-        <is>
-          <t>Matériel de connectivité (routeurs Wi-Fi, dongles 4G régions rurales)</t>
-        </is>
-      </c>
-      <c r="B17" s="38" t="inlineStr">
-        <is>
-          <t>Forfait — 14 régions à faible infrastructure</t>
-        </is>
-      </c>
-      <c r="C17" s="39" t="inlineStr">
-        <is>
-          <t>forfait</t>
-        </is>
-      </c>
-      <c r="D17" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="41" t="n">
-        <v>533</v>
-      </c>
-      <c r="F17" s="42" t="n">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Équipement et logiciels</t>
-        </is>
-      </c>
-      <c r="E18" s="44" t="n">
-        <v>8000</v>
-      </c>
-      <c r="F18" s="17" t="inlineStr">
-        <is>
-          <t>3.8%</t>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>3.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>3. COLLECTE ET TRAITEMENT DE DONNÉES</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="30" t="inlineStr">
-        <is>
-          <t>3. COLLECTE ET TRAITEMENT DE DONNÉES</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="31" t="inlineStr">
-        <is>
-          <t>14 coordinateurs locaux de collecte terrain</t>
-        </is>
-      </c>
-      <c r="B20" s="32" t="inlineStr">
-        <is>
-          <t>100 × 14 pers. × 8 mois actifs</t>
-        </is>
-      </c>
-      <c r="C20" s="33" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>54 collecteurs terrain — 3 par dialecte × 18 dialectes (recrutés dans les communautés, priorité aux femmes, rémunération équitable)</t>
+        </is>
+      </c>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>133 USD (600 000 MGA) × 54 pers. × 4 mois actifs</t>
+        </is>
+      </c>
+      <c r="C19" s="33" t="inlineStr">
         <is>
           <t>pers.×mois</t>
         </is>
       </c>
-      <c r="D20" s="34" t="n">
-        <v>112</v>
-      </c>
-      <c r="E20" s="35" t="n">
-        <v>100</v>
-      </c>
-      <c r="F20" s="36" t="n">
-        <v>11200</v>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Collecte et traitement de données</t>
-        </is>
-      </c>
-      <c r="E21" s="44" t="n">
-        <v>11200</v>
-      </c>
-      <c r="F21" s="17" t="inlineStr">
-        <is>
-          <t>5.3%</t>
+      <c r="D19" s="34" t="n">
+        <v>216</v>
+      </c>
+      <c r="E19" s="35" t="n">
+        <v>133</v>
+      </c>
+      <c r="F19" s="36" t="n">
+        <v>28728</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Collecte terrain</t>
+        </is>
+      </c>
+      <c r="E20" s="44" t="n">
+        <v>28728</v>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>4. ANNOTATION ET VÉRIFICATION (GROUND TRUTH)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="30" t="inlineStr">
-        <is>
-          <t>4. DÉPLACEMENTS ET TERRAIN</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="31" t="inlineStr">
-        <is>
-          <t>Missions régionales — avions intérieurs + taxi-brousse (14 régions, 2 visites)</t>
-        </is>
-      </c>
-      <c r="B23" s="32" t="inlineStr">
-        <is>
-          <t>400 × 14 régions × 2 allers-retours</t>
-        </is>
-      </c>
-      <c r="C23" s="33" t="inlineStr">
-        <is>
-          <t>mission</t>
-        </is>
-      </c>
-      <c r="D23" s="34" t="n">
-        <v>28</v>
-      </c>
-      <c r="E23" s="35" t="n">
-        <v>400</v>
-      </c>
-      <c r="F23" s="36" t="n">
-        <v>11200</v>
+      <c r="A22" s="31" t="inlineStr">
+        <is>
+          <t>36 annotateurs-transcripteurs — 2 par dialecte × 18 dialectes (vérification des transcriptions, alignement phonème-graphème, contrôle qualité)</t>
+        </is>
+      </c>
+      <c r="B22" s="32" t="inlineStr">
+        <is>
+          <t>200 USD (900 000 MGA) × 36 pers. × 4 mois actifs</t>
+        </is>
+      </c>
+      <c r="C22" s="33" t="inlineStr">
+        <is>
+          <t>pers.×mois</t>
+        </is>
+      </c>
+      <c r="D22" s="34" t="n">
+        <v>144</v>
+      </c>
+      <c r="E22" s="35" t="n">
+        <v>200</v>
+      </c>
+      <c r="F22" s="36" t="n">
+        <v>28800</v>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Annotation et ground truth</t>
+        </is>
+      </c>
+      <c r="E23" s="44" t="n">
+        <v>28800</v>
+      </c>
+      <c r="F23" s="17" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="37" t="inlineStr">
-        <is>
-          <t>Per diem et hébergement — superviseurs terrain</t>
-        </is>
-      </c>
-      <c r="B24" s="38" t="inlineStr">
-        <is>
-          <t>50/j × 3 j × 14 régions × 2 visites</t>
-        </is>
-      </c>
-      <c r="C24" s="39" t="inlineStr">
-        <is>
-          <t>j×mission</t>
-        </is>
-      </c>
-      <c r="D24" s="40" t="n">
-        <v>84</v>
-      </c>
-      <c r="E24" s="41" t="n">
-        <v>50</v>
-      </c>
-      <c r="F24" s="42" t="n">
-        <v>4200</v>
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>5. DÉPLACEMENTS ET TERRAIN</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="31" t="inlineStr">
         <is>
-          <t>Location de salles communautaires pour les sessions de collecte</t>
+          <t>Missions régionales — avions intérieurs + taxi-brousse (14 régions, 2 visites)</t>
         </is>
       </c>
       <c r="B25" s="32" t="inlineStr">
         <is>
-          <t>43 × 14 régions × 2 sessions  +  réserve imprévus</t>
+          <t>400 × 14 régions × 2 allers-retours</t>
         </is>
       </c>
       <c r="C25" s="33" t="inlineStr">
         <is>
-          <t>session</t>
+          <t>mission</t>
         </is>
       </c>
       <c r="D25" s="34" t="n">
         <v>28</v>
       </c>
       <c r="E25" s="35" t="n">
+        <v>400</v>
+      </c>
+      <c r="F25" s="36" t="n">
+        <v>11200</v>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="37" t="inlineStr">
+        <is>
+          <t>Per diem et hébergement — superviseurs terrain</t>
+        </is>
+      </c>
+      <c r="B26" s="38" t="inlineStr">
+        <is>
+          <t>50/j × 3 j × 14 régions × 2 visites</t>
+        </is>
+      </c>
+      <c r="C26" s="39" t="inlineStr">
+        <is>
+          <t>j×mission</t>
+        </is>
+      </c>
+      <c r="D26" s="40" t="n">
+        <v>84</v>
+      </c>
+      <c r="E26" s="41" t="n">
+        <v>50</v>
+      </c>
+      <c r="F26" s="42" t="n">
+        <v>4200</v>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="31" t="inlineStr">
+        <is>
+          <t>Location de salles communautaires pour les sessions de collecte</t>
+        </is>
+      </c>
+      <c r="B27" s="32" t="inlineStr">
+        <is>
+          <t>43 × 14 régions × 2 sessions  +  réserve imprévus</t>
+        </is>
+      </c>
+      <c r="C27" s="33" t="inlineStr">
+        <is>
+          <t>session</t>
+        </is>
+      </c>
+      <c r="D27" s="34" t="n">
+        <v>28</v>
+      </c>
+      <c r="E27" s="35" t="n">
         <v>43</v>
       </c>
-      <c r="F25" s="36" t="n">
+      <c r="F27" s="36" t="n">
         <v>600</v>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="43" t="inlineStr">
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="43" t="inlineStr">
         <is>
           <t>Sous-total Déplacements &amp; terrain</t>
         </is>
       </c>
-      <c r="E26" s="44" t="n">
+      <c r="E28" s="44" t="n">
         <v>16000</v>
       </c>
-      <c r="F26" s="17" t="inlineStr">
-        <is>
-          <t>7.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="30" t="inlineStr">
-        <is>
-          <t>5. FORMATION ET ATELIERS</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="31" t="inlineStr">
-        <is>
-          <t>Formation des 14 coordinateurs locaux (protocoles, outils d'enregistrement)</t>
-        </is>
-      </c>
-      <c r="B28" s="32" t="inlineStr">
-        <is>
-          <t>Salle + matériel + indemnités — 2 jours</t>
-        </is>
-      </c>
-      <c r="C28" s="33" t="inlineStr">
-        <is>
-          <t>forfait</t>
-        </is>
-      </c>
-      <c r="D28" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="35" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F28" s="36" t="n">
-        <v>1500</v>
+      <c r="F28" s="17" t="inlineStr">
+        <is>
+          <t>6.9%</t>
+        </is>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="37" t="inlineStr">
-        <is>
-          <t>Atelier de restitution final — communauté NLP africaine</t>
-        </is>
-      </c>
-      <c r="B29" s="38" t="inlineStr">
-        <is>
-          <t>Organisation, accueil participants, matériel de présentation</t>
-        </is>
-      </c>
-      <c r="C29" s="39" t="inlineStr">
-        <is>
-          <t>forfait</t>
-        </is>
-      </c>
-      <c r="D29" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="41" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F29" s="42" t="n">
-        <v>2000</v>
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>6. FORMATION ET ATELIERS</t>
+        </is>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="31" t="inlineStr">
         <is>
-          <t>Participation à une conférence NLP régionale (ex. IndabaX)</t>
+          <t>Formation des 14 coordinateurs locaux (protocoles, outils d'enregistrement)</t>
         </is>
       </c>
       <c r="B30" s="32" t="inlineStr">
         <is>
-          <t>Inscription + transport + hébergement</t>
+          <t>Salle + matériel + indemnités — 2 jours</t>
         </is>
       </c>
       <c r="C30" s="33" t="inlineStr">
@@ -1814,288 +1773,288 @@
         <v>1</v>
       </c>
       <c r="E30" s="35" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F30" s="36" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="37" t="inlineStr">
+        <is>
+          <t>Atelier de restitution final — communauté NLP africaine</t>
+        </is>
+      </c>
+      <c r="B31" s="38" t="inlineStr">
+        <is>
+          <t>Organisation, accueil participants, matériel de présentation</t>
+        </is>
+      </c>
+      <c r="C31" s="39" t="inlineStr">
+        <is>
+          <t>forfait</t>
+        </is>
+      </c>
+      <c r="D31" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="41" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F31" s="42" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="31" t="inlineStr">
+        <is>
+          <t>Participation à une conférence NLP régionale (ex. IndabaX)</t>
+        </is>
+      </c>
+      <c r="B32" s="32" t="inlineStr">
+        <is>
+          <t>Inscription + transport + hébergement</t>
+        </is>
+      </c>
+      <c r="C32" s="33" t="inlineStr">
+        <is>
+          <t>forfait</t>
+        </is>
+      </c>
+      <c r="D32" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="35" t="n">
         <v>1000</v>
       </c>
-      <c r="F30" s="36" t="n">
+      <c r="F32" s="36" t="n">
         <v>1000</v>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="43" t="inlineStr">
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="43" t="inlineStr">
         <is>
           <t>Sous-total Formation &amp; ateliers</t>
         </is>
       </c>
-      <c r="E31" s="44" t="n">
+      <c r="E33" s="44" t="n">
         <v>4500</v>
       </c>
-      <c r="F31" s="17" t="inlineStr">
-        <is>
-          <t>2.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="30" t="inlineStr">
-        <is>
-          <t>6. COMMUNICATION ET DOCUMENTATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="31" t="inlineStr">
+      <c r="F33" s="17" t="inlineStr">
+        <is>
+          <t>1.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>7. COMMUNICATION ET DOCUMENTATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="31" t="inlineStr">
         <is>
           <t>Rapports d'avancement semestriels (mise en page, traduction FR/EN)</t>
         </is>
       </c>
-      <c r="B33" s="32" t="inlineStr">
+      <c r="B35" s="32" t="inlineStr">
         <is>
           <t>250 × 6 rapports (M3, M6, M9, M12, M15, M18)</t>
         </is>
       </c>
-      <c r="C33" s="33" t="inlineStr">
+      <c r="C35" s="33" t="inlineStr">
         <is>
           <t>rapport</t>
         </is>
       </c>
-      <c r="D33" s="34" t="n">
+      <c r="D35" s="34" t="n">
         <v>6</v>
       </c>
-      <c r="E33" s="35" t="n">
+      <c r="E35" s="35" t="n">
         <v>100</v>
       </c>
-      <c r="F33" s="36" t="n">
+      <c r="F35" s="36" t="n">
         <v>600</v>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="37" t="inlineStr">
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="37" t="inlineStr">
         <is>
           <t>Outils numériques : gestion projet, hébergement web, licences</t>
         </is>
       </c>
-      <c r="B34" s="38" t="inlineStr">
+      <c r="B36" s="38" t="inlineStr">
         <is>
           <t>50/mois × 18 mois</t>
         </is>
       </c>
-      <c r="C34" s="39" t="inlineStr">
+      <c r="C36" s="39" t="inlineStr">
         <is>
           <t>mois</t>
         </is>
       </c>
-      <c r="D34" s="40" t="n">
+      <c r="D36" s="40" t="n">
         <v>18</v>
       </c>
-      <c r="E34" s="41" t="n">
+      <c r="E36" s="41" t="n">
         <v>50</v>
       </c>
-      <c r="F34" s="42" t="n">
+      <c r="F36" s="42" t="n">
         <v>900</v>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="43" t="inlineStr">
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="43" t="inlineStr">
         <is>
           <t>Sous-total Communication</t>
         </is>
       </c>
-      <c r="E35" s="44" t="n">
+      <c r="E37" s="44" t="n">
         <v>1500</v>
       </c>
-      <c r="F35" s="17" t="inlineStr">
-        <is>
-          <t>0.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="30" t="inlineStr">
-        <is>
-          <t>7. AUTRES COÛTS DIRECTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="31" t="inlineStr">
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>0.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
+          <t>8. AUTRES COÛTS DIRECTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="31" t="inlineStr">
         <is>
           <t>Frais administratifs et juridiques (contrats, enregistrements officiels)</t>
         </is>
       </c>
-      <c r="B37" s="32" t="inlineStr">
+      <c r="B39" s="32" t="inlineStr">
         <is>
           <t>Notaire, administration, légalisation</t>
         </is>
       </c>
-      <c r="C37" s="33" t="inlineStr">
+      <c r="C39" s="33" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D37" s="34" t="n">
+      <c r="D39" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="E37" s="35" t="n">
+      <c r="E39" s="35" t="n">
         <v>500</v>
       </c>
-      <c r="F37" s="36" t="n">
+      <c r="F39" s="36" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="37" t="inlineStr">
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="37" t="inlineStr">
         <is>
           <t>Réserve pour imprévus opérationnels</t>
         </is>
       </c>
-      <c r="B38" s="38" t="inlineStr">
+      <c r="B40" s="38" t="inlineStr">
         <is>
           <t>Ajustements terrain non anticipés</t>
         </is>
       </c>
-      <c r="C38" s="39" t="inlineStr">
+      <c r="C40" s="39" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D38" s="40" t="n">
+      <c r="D40" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E38" s="41" t="n">
+      <c r="E40" s="41" t="n">
         <v>500</v>
       </c>
-      <c r="F38" s="42" t="n">
+      <c r="F40" s="42" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="43" t="inlineStr">
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="43" t="inlineStr">
         <is>
           <t>Sous-total Autres coûts directs</t>
         </is>
       </c>
-      <c r="E39" s="44" t="n">
+      <c r="E41" s="44" t="n">
         <v>1000</v>
       </c>
-      <c r="F39" s="17" t="inlineStr">
-        <is>
-          <t>0.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="24" customHeight="1">
-      <c r="A40" s="45" t="inlineStr">
+      <c r="F41" s="17" t="inlineStr">
+        <is>
+          <t>0.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="24" customHeight="1">
+      <c r="A42" s="46" t="inlineStr">
         <is>
           <t>TOTAL DES COÛTS DIRECTS</t>
         </is>
       </c>
-      <c r="E40" s="46" t="n">
-        <v>209500</v>
-      </c>
-      <c r="F40" s="47" t="inlineStr">
+      <c r="E42" s="47" t="n">
+        <v>233428</v>
+      </c>
+      <c r="F42" s="48" t="inlineStr">
         <is>
           <t>100 %</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="43" t="inlineStr">
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="43" t="inlineStr">
         <is>
           <t>Frais généraux / Coûts indirects (5 % des coûts directs)</t>
         </is>
       </c>
-      <c r="E41" s="44" t="n">
-        <v>10500</v>
-      </c>
-      <c r="F41" s="48" t="inlineStr">
-        <is>
-          <t>5 % × 209 500</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="28" customHeight="1">
-      <c r="A42" s="18" t="inlineStr">
+      <c r="E43" s="44" t="n">
+        <v>11671</v>
+      </c>
+      <c r="F43" s="49" t="inlineStr">
+        <is>
+          <t>5 % × 233 428</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="28" customHeight="1">
+      <c r="A44" s="18" t="inlineStr">
         <is>
           <t>GRAND TOTAL — BUDGET CASH DEMANDÉ  (plafond Cat. 3 : 250 000 USD)</t>
         </is>
       </c>
-      <c r="E42" s="49" t="n">
-        <v>220000</v>
-      </c>
-      <c r="F42" s="50" t="inlineStr">
+      <c r="E44" s="50" t="n">
+        <v>245099</v>
+      </c>
+      <c r="F44" s="51" t="inlineStr">
         <is>
           <t>&lt; 250 000 USD ✓</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="51" t="inlineStr">
-        <is>
-          <t>8. RESSOURCES DE CALCUL GCP — Q18  (crédits séparés du budget cash — plafond 400 000 USD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="31" t="inlineStr">
-        <is>
-          <t>Vertex AI Custom Training — fine-tuning NLLB LoRA (6 langues × 18 dialectes)</t>
-        </is>
-      </c>
-      <c r="B45" s="32" t="inlineStr">
-        <is>
-          <t>L4 Spot ~0,28 $/h — expérimentations + runs finaux</t>
-        </is>
-      </c>
-      <c r="C45" s="33" t="inlineStr">
-        <is>
-          <t>forfait</t>
-        </is>
-      </c>
-      <c r="D45" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E45" s="35" t="n">
-        <v>45000</v>
-      </c>
-      <c r="F45" s="36" t="n">
-        <v>45000</v>
-      </c>
-    </row>
     <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="37" t="inlineStr">
-        <is>
-          <t>Vertex AI Custom Training — fine-tuning MMS-TTS VITS (18 dialectes)</t>
-        </is>
-      </c>
-      <c r="B46" s="38" t="inlineStr">
-        <is>
-          <t>18 dialectes × 3 cycles × 1,5 h GPU + hyperparamètres</t>
-        </is>
-      </c>
-      <c r="C46" s="39" t="inlineStr">
-        <is>
-          <t>forfait</t>
-        </is>
-      </c>
-      <c r="D46" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E46" s="41" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F46" s="42" t="n">
-        <v>20000</v>
+      <c r="A46" s="52" t="inlineStr">
+        <is>
+          <t>9. RESSOURCES DE CALCUL GCP — Q18  (crédits séparés du budget cash — plafond 400 000 USD)</t>
+        </is>
       </c>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="31" t="inlineStr">
         <is>
-          <t>Vertex AI Custom Training — buffer expérimentation &amp; réentraînement</t>
+          <t>Vertex AI Custom Training — fine-tuning NLLB LoRA (6 langues × 18 dialectes)</t>
         </is>
       </c>
       <c r="B47" s="32" t="inlineStr">
         <is>
-          <t>Nouvelles données M10–M18, réentraînements itératifs</t>
+          <t>L4 Spot ~0,28 $/h — expérimentations + runs finaux</t>
         </is>
       </c>
       <c r="C47" s="33" t="inlineStr">
@@ -2107,47 +2066,47 @@
         <v>1</v>
       </c>
       <c r="E47" s="35" t="n">
-        <v>15000</v>
+        <v>45000</v>
       </c>
       <c r="F47" s="36" t="n">
-        <v>15000</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="37" t="inlineStr">
         <is>
-          <t>Cloud Run GPU (NVIDIA L4 24 Go) — API MGVaovao en production</t>
+          <t>Vertex AI Custom Training — fine-tuning MMS-TTS VITS (18 dialectes)</t>
         </is>
       </c>
       <c r="B48" s="38" t="inlineStr">
         <is>
-          <t>~2 500 $/mois × 18 mois — scale-to-zero hors heures</t>
+          <t>18 dialectes × 3 cycles × 1,5 h GPU + hyperparamètres</t>
         </is>
       </c>
       <c r="C48" s="39" t="inlineStr">
         <is>
-          <t>mois</t>
+          <t>forfait</t>
         </is>
       </c>
       <c r="D48" s="40" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E48" s="41" t="n">
-        <v>2500</v>
+        <v>20000</v>
       </c>
       <c r="F48" s="42" t="n">
-        <v>45000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="31" t="inlineStr">
         <is>
-          <t>GCS — stockage corpus audio + checkpoints (≈ 3 To)</t>
+          <t>Vertex AI Custom Training — buffer expérimentation &amp; réentraînement</t>
         </is>
       </c>
       <c r="B49" s="32" t="inlineStr">
         <is>
-          <t>0,02 $/Go/mois × 3 000 Go × 18 mois + egress</t>
+          <t>Nouvelles données M10–M18, réentraînements itératifs</t>
         </is>
       </c>
       <c r="C49" s="33" t="inlineStr">
@@ -2159,73 +2118,73 @@
         <v>1</v>
       </c>
       <c r="E49" s="35" t="n">
-        <v>1500</v>
+        <v>15000</v>
       </c>
       <c r="F49" s="36" t="n">
-        <v>1500</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="37" t="inlineStr">
         <is>
-          <t>Vertex AI Pipelines — orchestration MLOps Kubeflow DAG</t>
+          <t>Cloud Run GPU (NVIDIA L4 24 Go) — API MGVaovao en production</t>
         </is>
       </c>
       <c r="B50" s="38" t="inlineStr">
         <is>
-          <t>0,03 $/run × ~500 runs + monitoring continu</t>
+          <t>~2 500 $/mois × 18 mois — scale-to-zero hors heures</t>
         </is>
       </c>
       <c r="C50" s="39" t="inlineStr">
         <is>
-          <t>forfait</t>
+          <t>mois</t>
         </is>
       </c>
       <c r="D50" s="40" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="E50" s="41" t="n">
-        <v>500</v>
+        <v>2500</v>
       </c>
       <c r="F50" s="42" t="n">
-        <v>500</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="31" t="inlineStr">
         <is>
-          <t>Cloud Build, Artifact Registry, Cloud Monitoring, Pub/Sub</t>
+          <t>GCS — stockage corpus audio + checkpoints (≈ 3 To)</t>
         </is>
       </c>
       <c r="B51" s="32" t="inlineStr">
         <is>
-          <t>CI/CD, registre d'images, alertes, déclencheurs GCS</t>
+          <t>0,02 $/Go/mois × 3 000 Go × 18 mois + egress</t>
         </is>
       </c>
       <c r="C51" s="33" t="inlineStr">
         <is>
-          <t>mois</t>
+          <t>forfait</t>
         </is>
       </c>
       <c r="D51" s="34" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E51" s="35" t="n">
-        <v>139</v>
+        <v>1500</v>
       </c>
       <c r="F51" s="36" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="37" t="inlineStr">
         <is>
-          <t>Dataflow / ingestion pipeline audio — traitement et normalisation</t>
+          <t>Vertex AI Pipelines — orchestration MLOps Kubeflow DAG</t>
         </is>
       </c>
       <c r="B52" s="38" t="inlineStr">
         <is>
-          <t>Ingestion et prétraitement audio en pipeline GCS</t>
+          <t>0,03 $/run × ~500 runs + monitoring continu</t>
         </is>
       </c>
       <c r="C52" s="39" t="inlineStr">
@@ -2237,49 +2196,104 @@
         <v>1</v>
       </c>
       <c r="E52" s="41" t="n">
+        <v>500</v>
+      </c>
+      <c r="F52" s="42" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="31" t="inlineStr">
+        <is>
+          <t>Cloud Build, Artifact Registry, Cloud Monitoring, Pub/Sub</t>
+        </is>
+      </c>
+      <c r="B53" s="32" t="inlineStr">
+        <is>
+          <t>CI/CD, registre d'images, alertes, déclencheurs GCS</t>
+        </is>
+      </c>
+      <c r="C53" s="33" t="inlineStr">
+        <is>
+          <t>mois</t>
+        </is>
+      </c>
+      <c r="D53" s="34" t="n">
+        <v>18</v>
+      </c>
+      <c r="E53" s="35" t="n">
+        <v>139</v>
+      </c>
+      <c r="F53" s="36" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="37" t="inlineStr">
+        <is>
+          <t>Dataflow / ingestion pipeline audio — traitement et normalisation</t>
+        </is>
+      </c>
+      <c r="B54" s="38" t="inlineStr">
+        <is>
+          <t>Ingestion et prétraitement audio en pipeline GCS</t>
+        </is>
+      </c>
+      <c r="C54" s="39" t="inlineStr">
+        <is>
+          <t>forfait</t>
+        </is>
+      </c>
+      <c r="D54" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="41" t="n">
         <v>20500</v>
       </c>
-      <c r="F52" s="42" t="n">
+      <c r="F54" s="42" t="n">
         <v>20500</v>
       </c>
     </row>
-    <row r="53" ht="28" customHeight="1">
-      <c r="A53" s="21" t="inlineStr">
+    <row r="55" ht="28" customHeight="1">
+      <c r="A55" s="21" t="inlineStr">
         <is>
           <t>TOTAL CRÉDITS GCP DEMANDÉS  (Q18b — séparé du budget cash)</t>
         </is>
       </c>
-      <c r="E53" s="52" t="n">
+      <c r="E55" s="53" t="n">
         <v>150000</v>
       </c>
-      <c r="F53" s="53" t="inlineStr">
+      <c r="F55" s="54" t="inlineStr">
         <is>
           <t>&lt; 400 000 USD ✓</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A27:F27"/>
+  <mergeCells count="24">
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A44:D44"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A39:D39"/>
-    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A34:F34"/>
     <mergeCell ref="A41:D41"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A37:D37"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A55:D55"/>
+    <mergeCell ref="A33:D33"/>
     <mergeCell ref="A42:D42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2292,7 +2306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2302,323 +2316,343 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="54" t="inlineStr">
+      <c r="A1" s="55" t="inlineStr">
         <is>
           <t>RÉSUMÉ BUDGÉTAIRE — MGVaovao / LINGUA AFRICA 2026</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="55" t="inlineStr">
+      <c r="A2" s="56" t="inlineStr">
         <is>
           <t>Catégorie 3 — Applications sectorielles  |  Budget cash ≤ 250 000 USD  +  Crédits GCP ≤ 400 000 USD</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="56" t="inlineStr">
+      <c r="A3" s="57" t="inlineStr">
         <is>
           <t>Catégorie de coût</t>
         </is>
       </c>
-      <c r="B3" s="56" t="inlineStr">
+      <c r="B3" s="57" t="inlineStr">
         <is>
           <t>Montant (USD)</t>
         </is>
       </c>
-      <c r="C3" s="56" t="inlineStr">
+      <c r="C3" s="57" t="inlineStr">
         <is>
           <t>% coûts directs</t>
         </is>
       </c>
-      <c r="D3" s="56" t="inlineStr">
+      <c r="D3" s="57" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="57" t="inlineStr">
-        <is>
-          <t>1. Personnel</t>
-        </is>
-      </c>
-      <c r="B4" s="58" t="n">
-        <v>167300</v>
-      </c>
-      <c r="C4" s="59" t="inlineStr">
-        <is>
-          <t>79.9 %</t>
-        </is>
-      </c>
-      <c r="D4" s="59" t="inlineStr">
-        <is>
-          <t>Équipe permanente 18 mois — 7 postes</t>
+      <c r="A4" s="58" t="inlineStr">
+        <is>
+          <t>1. Personnel — direction permanente</t>
+        </is>
+      </c>
+      <c r="B4" s="59" t="n">
+        <v>144900</v>
+      </c>
+      <c r="C4" s="60" t="inlineStr">
+        <is>
+          <t>62.1 %</t>
+        </is>
+      </c>
+      <c r="D4" s="60" t="inlineStr">
+        <is>
+          <t>5 postes : direction, ML, data ops, partenariats — 18 mois</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="60" t="inlineStr">
+      <c r="A5" s="61" t="inlineStr">
         <is>
           <t>2. Équipement et logiciels</t>
         </is>
       </c>
-      <c r="B5" s="61" t="n">
+      <c r="B5" s="62" t="n">
         <v>8000</v>
       </c>
-      <c r="C5" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 3.8 %</t>
-        </is>
-      </c>
-      <c r="D5" s="62" t="inlineStr">
-        <is>
-          <t>Laptops, tablettes, micros, connectivité</t>
+      <c r="C5" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 3.4 %</t>
+        </is>
+      </c>
+      <c r="D5" s="63" t="inlineStr">
+        <is>
+          <t>Laptops, matériel d'enregistrement terrain, connectivité</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="57" t="inlineStr">
-        <is>
-          <t>3. Collecte et traitement de données</t>
-        </is>
-      </c>
-      <c r="B6" s="58" t="n">
-        <v>11200</v>
-      </c>
-      <c r="C6" s="59" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 5.3 %</t>
-        </is>
-      </c>
-      <c r="D6" s="59" t="inlineStr">
-        <is>
-          <t>14 coordinateurs locaux terrain × 8 mois × 100 USD</t>
+      <c r="A6" s="58" t="inlineStr">
+        <is>
+          <t>3. Collecte terrain</t>
+        </is>
+      </c>
+      <c r="B6" s="59" t="n">
+        <v>28728</v>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>12.3 %</t>
+        </is>
+      </c>
+      <c r="D6" s="60" t="inlineStr">
+        <is>
+          <t>54 collecteurs × 133 USD/mois × 4 mois — 3 par dialecte × 18</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="60" t="inlineStr">
-        <is>
-          <t>4. Déplacements et terrain</t>
-        </is>
-      </c>
-      <c r="B7" s="61" t="n">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>4. Annotation et ground truth</t>
+        </is>
+      </c>
+      <c r="B7" s="62" t="n">
+        <v>28800</v>
+      </c>
+      <c r="C7" s="63" t="inlineStr">
+        <is>
+          <t>12.3 %</t>
+        </is>
+      </c>
+      <c r="D7" s="63" t="inlineStr">
+        <is>
+          <t>36 annotateurs × 200 USD/mois × 4 mois — 2 par dialecte × 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="58" t="inlineStr">
+        <is>
+          <t>5. Déplacements et terrain</t>
+        </is>
+      </c>
+      <c r="B8" s="59" t="n">
         <v>16000</v>
       </c>
-      <c r="C7" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 7.6 %</t>
-        </is>
-      </c>
-      <c r="D7" s="62" t="inlineStr">
-        <is>
-          <t>14 régions × 2 missions — avion + taxi-brousse</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="57" t="inlineStr">
-        <is>
-          <t>5. Formation et ateliers</t>
-        </is>
-      </c>
-      <c r="B8" s="58" t="n">
+      <c r="C8" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6.9 %</t>
+        </is>
+      </c>
+      <c r="D8" s="60" t="inlineStr">
+        <is>
+          <t>18 régions × 2 missions — avion, per diem, salles</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>6. Formation et ateliers</t>
+        </is>
+      </c>
+      <c r="B9" s="62" t="n">
         <v>4500</v>
       </c>
-      <c r="C8" s="59" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 2.1 %</t>
-        </is>
-      </c>
-      <c r="D8" s="59" t="inlineStr">
-        <is>
-          <t>Formation coordinateurs + atelier restitution + conférence</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="60" t="inlineStr">
-        <is>
-          <t>6. Communication et documentation</t>
-        </is>
-      </c>
-      <c r="B9" s="61" t="n">
+      <c r="C9" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1.9 %</t>
+        </is>
+      </c>
+      <c r="D9" s="63" t="inlineStr">
+        <is>
+          <t>Formation équipes terrain + atelier restitution + conférence</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="58" t="inlineStr">
+        <is>
+          <t>7. Communication et documentation</t>
+        </is>
+      </c>
+      <c r="B10" s="59" t="n">
         <v>1500</v>
       </c>
-      <c r="C9" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 0.7 %</t>
-        </is>
-      </c>
-      <c r="D9" s="62" t="inlineStr">
-        <is>
-          <t>Rapports, outils numériques</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="57" t="inlineStr">
-        <is>
-          <t>7. Autres coûts directs</t>
-        </is>
-      </c>
-      <c r="B10" s="58" t="n">
+      <c r="C10" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 0.6 %</t>
+        </is>
+      </c>
+      <c r="D10" s="60" t="inlineStr">
+        <is>
+          <t>Rapports semestriels, outils numériques</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>8. Autres coûts directs</t>
+        </is>
+      </c>
+      <c r="B11" s="62" t="n">
         <v>1000</v>
       </c>
-      <c r="C10" s="59" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 0.5 %</t>
-        </is>
-      </c>
-      <c r="D10" s="59" t="inlineStr">
+      <c r="C11" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 0.4 %</t>
+        </is>
+      </c>
+      <c r="D11" s="63" t="inlineStr">
         <is>
           <t>Frais administratifs + réserve imprévus</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="63" t="inlineStr">
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="64" t="inlineStr">
         <is>
           <t>TOTAL DES COÛTS DIRECTS</t>
         </is>
       </c>
-      <c r="B11" s="46" t="n">
-        <v>209500</v>
-      </c>
-      <c r="C11" s="47" t="inlineStr">
+      <c r="B12" s="47" t="n">
+        <v>233428</v>
+      </c>
+      <c r="C12" s="48" t="inlineStr">
         <is>
           <t>100 %</t>
         </is>
       </c>
-      <c r="D11" s="47" t="inlineStr">
+      <c r="D12" s="48" t="inlineStr">
         <is>
           <t>209 500 USD</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="64" t="inlineStr">
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="65" t="inlineStr">
         <is>
           <t>Frais généraux / indirects (5 %)</t>
         </is>
       </c>
-      <c r="B12" s="44" t="n">
-        <v>10500</v>
-      </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="B13" s="44" t="n">
+        <v>11671</v>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>5 %</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
-        <is>
-          <t>5 % × 209 500</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="65" t="inlineStr">
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>5 % × 233 428</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="66" t="inlineStr">
         <is>
           <t>GRAND TOTAL — BUDGET CASH DEMANDÉ</t>
         </is>
       </c>
-      <c r="B13" s="49" t="n">
-        <v>220000</v>
-      </c>
-      <c r="C13" s="66" t="inlineStr">
+      <c r="B14" s="50" t="n">
+        <v>245099</v>
+      </c>
+      <c r="C14" s="67" t="inlineStr">
         <is>
           <t>&lt; 250 000 USD ✓</t>
         </is>
       </c>
-      <c r="D13" s="66" t="inlineStr">
+      <c r="D14" s="67" t="inlineStr">
         <is>
           <t>Plafond Cat. 3 respecté</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="67" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="68" t="inlineStr">
         <is>
           <t>RESSOURCES DE CALCUL GCP — Q18  (séparées du budget cash — plafond 400 000 USD)</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="57" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="58" t="inlineStr">
         <is>
           <t>Vertex AI Custom Training — NLLB LoRA + MMS-TTS + expérimentation</t>
         </is>
       </c>
-      <c r="B16" s="58" t="n">
+      <c r="B17" s="59" t="n">
         <v>80000</v>
       </c>
-      <c r="C16" s="59" t="inlineStr">
+      <c r="C17" s="60" t="inlineStr">
         <is>
           <t>53.3 %</t>
         </is>
       </c>
-      <c r="D16" s="59" t="inlineStr">
+      <c r="D17" s="60" t="inlineStr">
         <is>
           <t>6 langues × 18 dialectes + cycles itératifs</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="60" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="61" t="inlineStr">
         <is>
           <t>Cloud Run GPU — infrastructure de production API (18 mois)</t>
         </is>
       </c>
-      <c r="B17" s="61" t="n">
+      <c r="B18" s="62" t="n">
         <v>45000</v>
       </c>
-      <c r="C17" s="62" t="inlineStr">
+      <c r="C18" s="63" t="inlineStr">
         <is>
           <t>30.0 %</t>
         </is>
       </c>
-      <c r="D17" s="62" t="inlineStr">
+      <c r="D18" s="63" t="inlineStr">
         <is>
           <t>NVIDIA L4 24 Go — scale-to-zero hors heures</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="57" t="inlineStr">
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="58" t="inlineStr">
         <is>
           <t>GCS, Pipelines, CI/CD, Monitoring, Dataflow, Pub/Sub</t>
         </is>
       </c>
-      <c r="B18" s="58" t="n">
+      <c r="B19" s="59" t="n">
         <v>25000</v>
       </c>
-      <c r="C18" s="59" t="inlineStr">
+      <c r="C19" s="60" t="inlineStr">
         <is>
           <t>16.7 %</t>
         </is>
       </c>
-      <c r="D18" s="59" t="inlineStr">
+      <c r="D19" s="60" t="inlineStr">
         <is>
           <t>Stockage 3 To + orchestration MLOps + ingestion</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="68" t="inlineStr">
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="69" t="inlineStr">
         <is>
           <t>TOTAL CRÉDITS GCP DEMANDÉS (Q18b)</t>
         </is>
       </c>
-      <c r="B19" s="52" t="n">
+      <c r="B20" s="53" t="n">
         <v>150000</v>
       </c>
-      <c r="C19" s="69" t="inlineStr">
+      <c r="C20" s="70" t="inlineStr">
         <is>
           <t>&lt; 400 000 USD ✓</t>
         </is>
       </c>
-      <c r="D19" s="69" t="inlineStr">
+      <c r="D20" s="70" t="inlineStr">
         <is>
           <t>Plafond Q18 respecté</t>
         </is>
@@ -2627,8 +2661,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A16:D16"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A15:D15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Budget: integrate 8 devs fully, reduce data workers to stay within 250K cap
All 8 developers (1 500 000 MGA/month = 333 USD) are now inside the LINGUA
Africa budget. Personnel rises to 192 852 USD (13 posts). Data collection is
reduced to 20 collectors × 133 USD × 4 months (10 640 USD) and 9 annotators
× 133 USD × 3 months (3 591 USD) to respect the cap.

Grand total: 238 083 direct + 11 904 overhead = 249 987 USD (< 250 000 ✓).

Updated: generate_budget.py, generate_application.py, generate_application_en.py,
LINGUA_Africa_Application_QA.md and all three generated artefacts.
</commit_message>
<xml_diff>
--- a/LINGUA_Africa_Budget_Detaille.xlsx
+++ b/LINGUA_Africa_Budget_Detaille.xlsx
@@ -155,7 +155,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -195,11 +195,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F0F4F7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -248,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -378,16 +373,13 @@
     <xf numFmtId="3" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="15" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="15" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -435,7 +427,7 @@
     <xf numFmtId="0" fontId="22" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -899,15 +891,15 @@
       <c r="A9" s="1" t="inlineStr"/>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Personnel — direction permanente</t>
+          <t>Personnel — direction + équipe technique (13 postes)</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>144900</v>
+        <v>192852</v>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>62.1 % des coûts directs</t>
+          <t>81.0 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -931,15 +923,15 @@
       <c r="A11" s="1" t="inlineStr"/>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Collecte terrain (54 collecteurs)</t>
+          <t>Collecte terrain (20 collecteurs)</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>28728</v>
+        <v>10640</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>12.3 % des coûts directs</t>
+          <t xml:space="preserve"> 4.5 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -947,15 +939,15 @@
       <c r="A12" s="1" t="inlineStr"/>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Annotation ground truth (36 annotateurs)</t>
+          <t>Annotation ground truth (9 annotateurs)</t>
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>28800</v>
+        <v>3591</v>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>12.3 % des coûts directs</t>
+          <t xml:space="preserve"> 1.5 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -971,7 +963,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 6.9 % des coûts directs</t>
+          <t xml:space="preserve"> 6.7 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1007,7 @@
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>233428</v>
+        <v>238083</v>
       </c>
       <c r="D16" s="14" t="n"/>
     </row>
@@ -1030,11 +1022,11 @@
         </is>
       </c>
       <c r="C18" s="16" t="n">
-        <v>11671</v>
+        <v>11904</v>
       </c>
       <c r="D18" s="17" t="inlineStr">
         <is>
-          <t>5 % × 233 428</t>
+          <t>5 % × 238 083</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1038,7 @@
         </is>
       </c>
       <c r="C19" s="19" t="n">
-        <v>245099</v>
+        <v>249987</v>
       </c>
       <c r="D19" s="20" t="inlineStr">
         <is>
@@ -1208,7 +1200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1402,540 +1394,619 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Personnel (direction permanente)</t>
-        </is>
-      </c>
-      <c r="E10" s="44" t="n">
-        <v>144900</v>
-      </c>
-      <c r="F10" s="17" t="inlineStr">
-        <is>
-          <t>62.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="45" t="inlineStr">
-        <is>
-          <t>↳ Co-financement organisation (hors budget LINGUA Africa) : 8 développeurs (backend / frontend / IA / data science / DevOps) × 333 USD (1 500 000 MGA) × 18 mois = 47 952 USD</t>
-        </is>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="37" t="inlineStr">
+        <is>
+          <t>Développeur backend (100 %)</t>
+        </is>
+      </c>
+      <c r="B10" s="38" t="inlineStr">
+        <is>
+          <t>333 × 18 mois  ≈ 1 500 000 MGA/mois</t>
+        </is>
+      </c>
+      <c r="C10" s="39" t="inlineStr">
+        <is>
+          <t>mois</t>
+        </is>
+      </c>
+      <c r="D10" s="40" t="n">
+        <v>18</v>
+      </c>
+      <c r="E10" s="41" t="n">
+        <v>333</v>
+      </c>
+      <c r="F10" s="42" t="n">
+        <v>5994</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>Développeur frontend (100 %)</t>
+        </is>
+      </c>
+      <c r="B11" s="32" t="inlineStr">
+        <is>
+          <t>333 × 18 mois  ≈ 1 500 000 MGA/mois</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>mois</t>
+        </is>
+      </c>
+      <c r="D11" s="34" t="n">
+        <v>18</v>
+      </c>
+      <c r="E11" s="35" t="n">
+        <v>333</v>
+      </c>
+      <c r="F11" s="36" t="n">
+        <v>5994</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="30" t="inlineStr">
-        <is>
-          <t>2. ÉQUIPEMENT ET LOGICIELS</t>
-        </is>
+      <c r="A12" s="37" t="inlineStr">
+        <is>
+          <t>Développeur IA / ML engineer 1 (100 %)</t>
+        </is>
+      </c>
+      <c r="B12" s="38" t="inlineStr">
+        <is>
+          <t>333 × 18 mois  ≈ 1 500 000 MGA/mois</t>
+        </is>
+      </c>
+      <c r="C12" s="39" t="inlineStr">
+        <is>
+          <t>mois</t>
+        </is>
+      </c>
+      <c r="D12" s="40" t="n">
+        <v>18</v>
+      </c>
+      <c r="E12" s="41" t="n">
+        <v>333</v>
+      </c>
+      <c r="F12" s="42" t="n">
+        <v>5994</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="31" t="inlineStr">
         <is>
-          <t>Ordinateurs portables — équipe technique locale (hors fondateur à Zurich)</t>
+          <t>Développeur IA / ML engineer 2 (100 %)</t>
         </is>
       </c>
       <c r="B13" s="32" t="inlineStr">
         <is>
-          <t>778 USD × 6 unités  (≈ 3 500 000 MGA l'unité)</t>
+          <t>333 × 18 mois  ≈ 1 500 000 MGA/mois</t>
         </is>
       </c>
       <c r="C13" s="33" t="inlineStr">
         <is>
-          <t>unité</t>
+          <t>mois</t>
         </is>
       </c>
       <c r="D13" s="34" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="E13" s="35" t="n">
-        <v>778</v>
+        <v>333</v>
       </c>
       <c r="F13" s="36" t="n">
-        <v>4667</v>
+        <v>5994</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="37" t="inlineStr">
         <is>
-          <t>Tablettes de terrain pour coordinateurs de collecte</t>
+          <t>Data scientist / ML engineer (100 %)</t>
         </is>
       </c>
       <c r="B14" s="38" t="inlineStr">
         <is>
-          <t>150 × 14 coordinateurs</t>
+          <t>333 × 18 mois  ≈ 1 500 000 MGA/mois</t>
         </is>
       </c>
       <c r="C14" s="39" t="inlineStr">
         <is>
-          <t>unité</t>
+          <t>mois</t>
         </is>
       </c>
       <c r="D14" s="40" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E14" s="41" t="n">
-        <v>150</v>
+        <v>333</v>
       </c>
       <c r="F14" s="42" t="n">
-        <v>2100</v>
+        <v>5994</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="31" t="inlineStr">
         <is>
-          <t>Microphones USB qualité ASR/TTS pour les sessions de collecte</t>
+          <t>DevOps engineer (100 %)</t>
         </is>
       </c>
       <c r="B15" s="32" t="inlineStr">
         <is>
-          <t>50 × 14 coordinateurs</t>
+          <t>333 × 18 mois  ≈ 1 500 000 MGA/mois</t>
         </is>
       </c>
       <c r="C15" s="33" t="inlineStr">
         <is>
-          <t>unité</t>
+          <t>mois</t>
         </is>
       </c>
       <c r="D15" s="34" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E15" s="35" t="n">
-        <v>50</v>
+        <v>333</v>
       </c>
       <c r="F15" s="36" t="n">
-        <v>700</v>
+        <v>5994</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="37" t="inlineStr">
         <is>
-          <t>Matériel de connectivité (routeurs Wi-Fi, dongles 4G régions rurales)</t>
+          <t>Développeur full-stack (100 %)</t>
         </is>
       </c>
       <c r="B16" s="38" t="inlineStr">
         <is>
-          <t>Forfait — 14 régions à faible infrastructure</t>
+          <t>333 × 18 mois  ≈ 1 500 000 MGA/mois</t>
         </is>
       </c>
       <c r="C16" s="39" t="inlineStr">
         <is>
-          <t>forfait</t>
+          <t>mois</t>
         </is>
       </c>
       <c r="D16" s="40" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="E16" s="41" t="n">
-        <v>533</v>
+        <v>333</v>
       </c>
       <c r="F16" s="42" t="n">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Équipement et logiciels</t>
-        </is>
-      </c>
-      <c r="E17" s="44" t="n">
-        <v>8000</v>
-      </c>
-      <c r="F17" s="17" t="inlineStr">
-        <is>
-          <t>3.4%</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="30" t="inlineStr">
-        <is>
-          <t>3. COLLECTE ET TRAITEMENT DE DONNÉES</t>
+        <v>5994</v>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="31" t="inlineStr">
+        <is>
+          <t>Data engineer (100 %)</t>
+        </is>
+      </c>
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>333 × 18 mois  ≈ 1 500 000 MGA/mois</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="inlineStr">
+        <is>
+          <t>mois</t>
+        </is>
+      </c>
+      <c r="D17" s="34" t="n">
+        <v>18</v>
+      </c>
+      <c r="E17" s="35" t="n">
+        <v>333</v>
+      </c>
+      <c r="F17" s="36" t="n">
+        <v>5994</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Personnel (direction + équipe technique)</t>
+        </is>
+      </c>
+      <c r="E18" s="44" t="n">
+        <v>192852</v>
+      </c>
+      <c r="F18" s="17" t="inlineStr">
+        <is>
+          <t>81.0%</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="31" t="inlineStr">
-        <is>
-          <t>54 collecteurs terrain — 3 par dialecte × 18 dialectes (recrutés dans les communautés, priorité aux femmes, rémunération équitable)</t>
-        </is>
-      </c>
-      <c r="B19" s="32" t="inlineStr">
-        <is>
-          <t>133 USD (600 000 MGA) × 54 pers. × 4 mois actifs</t>
-        </is>
-      </c>
-      <c r="C19" s="33" t="inlineStr">
-        <is>
-          <t>pers.×mois</t>
-        </is>
-      </c>
-      <c r="D19" s="34" t="n">
-        <v>216</v>
-      </c>
-      <c r="E19" s="35" t="n">
-        <v>133</v>
-      </c>
-      <c r="F19" s="36" t="n">
-        <v>28728</v>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Collecte terrain</t>
-        </is>
-      </c>
-      <c r="E20" s="44" t="n">
-        <v>28728</v>
-      </c>
-      <c r="F20" s="17" t="inlineStr">
-        <is>
-          <t>12.3%</t>
-        </is>
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>2. ÉQUIPEMENT ET LOGICIELS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>Ordinateurs portables — équipe technique locale (hors fondateur à Zurich)</t>
+        </is>
+      </c>
+      <c r="B20" s="32" t="inlineStr">
+        <is>
+          <t>778 USD × 6 unités  (≈ 3 500 000 MGA l'unité)</t>
+        </is>
+      </c>
+      <c r="C20" s="33" t="inlineStr">
+        <is>
+          <t>unité</t>
+        </is>
+      </c>
+      <c r="D20" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E20" s="35" t="n">
+        <v>778</v>
+      </c>
+      <c r="F20" s="36" t="n">
+        <v>4667</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="30" t="inlineStr">
-        <is>
-          <t>4. ANNOTATION ET VÉRIFICATION (GROUND TRUTH)</t>
-        </is>
+      <c r="A21" s="37" t="inlineStr">
+        <is>
+          <t>Tablettes de terrain pour coordinateurs de collecte</t>
+        </is>
+      </c>
+      <c r="B21" s="38" t="inlineStr">
+        <is>
+          <t>150 × 14 coordinateurs</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="inlineStr">
+        <is>
+          <t>unité</t>
+        </is>
+      </c>
+      <c r="D21" s="40" t="n">
+        <v>14</v>
+      </c>
+      <c r="E21" s="41" t="n">
+        <v>150</v>
+      </c>
+      <c r="F21" s="42" t="n">
+        <v>2100</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="31" t="inlineStr">
         <is>
-          <t>36 annotateurs-transcripteurs — 2 par dialecte × 18 dialectes (vérification des transcriptions, alignement phonème-graphème, contrôle qualité)</t>
+          <t>Microphones USB qualité ASR/TTS pour les sessions de collecte</t>
         </is>
       </c>
       <c r="B22" s="32" t="inlineStr">
         <is>
-          <t>200 USD (900 000 MGA) × 36 pers. × 4 mois actifs</t>
+          <t>50 × 14 coordinateurs</t>
         </is>
       </c>
       <c r="C22" s="33" t="inlineStr">
         <is>
+          <t>unité</t>
+        </is>
+      </c>
+      <c r="D22" s="34" t="n">
+        <v>14</v>
+      </c>
+      <c r="E22" s="35" t="n">
+        <v>50</v>
+      </c>
+      <c r="F22" s="36" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="37" t="inlineStr">
+        <is>
+          <t>Matériel de connectivité (routeurs Wi-Fi, dongles 4G régions rurales)</t>
+        </is>
+      </c>
+      <c r="B23" s="38" t="inlineStr">
+        <is>
+          <t>Forfait — 14 régions à faible infrastructure</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>forfait</t>
+        </is>
+      </c>
+      <c r="D23" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="41" t="n">
+        <v>533</v>
+      </c>
+      <c r="F23" s="42" t="n">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Équipement et logiciels</t>
+        </is>
+      </c>
+      <c r="E24" s="44" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F24" s="17" t="inlineStr">
+        <is>
+          <t>3.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>3. COLLECTE ET TRAITEMENT DE DONNÉES</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="31" t="inlineStr">
+        <is>
+          <t>20 collecteurs terrain — 1 à 2 par dialecte × 18 dialectes (recrutés dans les communautés, priorité aux femmes, rémunération équitable)</t>
+        </is>
+      </c>
+      <c r="B26" s="32" t="inlineStr">
+        <is>
+          <t>133 USD (600 000 MGA) × 20 pers. × 4 mois actifs</t>
+        </is>
+      </c>
+      <c r="C26" s="33" t="inlineStr">
+        <is>
           <t>pers.×mois</t>
         </is>
       </c>
-      <c r="D22" s="34" t="n">
-        <v>144</v>
-      </c>
-      <c r="E22" s="35" t="n">
-        <v>200</v>
-      </c>
-      <c r="F22" s="36" t="n">
-        <v>28800</v>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="43" t="inlineStr">
+      <c r="D26" s="34" t="n">
+        <v>80</v>
+      </c>
+      <c r="E26" s="35" t="n">
+        <v>133</v>
+      </c>
+      <c r="F26" s="36" t="n">
+        <v>10640</v>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Collecte terrain</t>
+        </is>
+      </c>
+      <c r="E27" s="44" t="n">
+        <v>10640</v>
+      </c>
+      <c r="F27" s="17" t="inlineStr">
+        <is>
+          <t>4.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>4. ANNOTATION ET VÉRIFICATION (GROUND TRUTH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="31" t="inlineStr">
+        <is>
+          <t>9 annotateurs-transcripteurs — vérification des transcriptions, alignement phonème-graphème, contrôle qualité</t>
+        </is>
+      </c>
+      <c r="B29" s="32" t="inlineStr">
+        <is>
+          <t>133 USD (600 000 MGA) × 9 pers. × 3 mois actifs</t>
+        </is>
+      </c>
+      <c r="C29" s="33" t="inlineStr">
+        <is>
+          <t>pers.×mois</t>
+        </is>
+      </c>
+      <c r="D29" s="34" t="n">
+        <v>27</v>
+      </c>
+      <c r="E29" s="35" t="n">
+        <v>133</v>
+      </c>
+      <c r="F29" s="36" t="n">
+        <v>3591</v>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="43" t="inlineStr">
         <is>
           <t>Sous-total Annotation et ground truth</t>
         </is>
       </c>
-      <c r="E23" s="44" t="n">
-        <v>28800</v>
-      </c>
-      <c r="F23" s="17" t="inlineStr">
-        <is>
-          <t>12.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="30" t="inlineStr">
+      <c r="E30" s="44" t="n">
+        <v>3591</v>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>1.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="30" t="inlineStr">
         <is>
           <t>5. DÉPLACEMENTS ET TERRAIN</t>
         </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="31" t="inlineStr">
-        <is>
-          <t>Missions régionales — avions intérieurs + taxi-brousse (14 régions, 2 visites)</t>
-        </is>
-      </c>
-      <c r="B25" s="32" t="inlineStr">
-        <is>
-          <t>400 × 14 régions × 2 allers-retours</t>
-        </is>
-      </c>
-      <c r="C25" s="33" t="inlineStr">
-        <is>
-          <t>mission</t>
-        </is>
-      </c>
-      <c r="D25" s="34" t="n">
-        <v>28</v>
-      </c>
-      <c r="E25" s="35" t="n">
-        <v>400</v>
-      </c>
-      <c r="F25" s="36" t="n">
-        <v>11200</v>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="37" t="inlineStr">
-        <is>
-          <t>Per diem et hébergement — superviseurs terrain</t>
-        </is>
-      </c>
-      <c r="B26" s="38" t="inlineStr">
-        <is>
-          <t>50/j × 3 j × 14 régions × 2 visites</t>
-        </is>
-      </c>
-      <c r="C26" s="39" t="inlineStr">
-        <is>
-          <t>j×mission</t>
-        </is>
-      </c>
-      <c r="D26" s="40" t="n">
-        <v>84</v>
-      </c>
-      <c r="E26" s="41" t="n">
-        <v>50</v>
-      </c>
-      <c r="F26" s="42" t="n">
-        <v>4200</v>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="31" t="inlineStr">
-        <is>
-          <t>Location de salles communautaires pour les sessions de collecte</t>
-        </is>
-      </c>
-      <c r="B27" s="32" t="inlineStr">
-        <is>
-          <t>43 × 14 régions × 2 sessions  +  réserve imprévus</t>
-        </is>
-      </c>
-      <c r="C27" s="33" t="inlineStr">
-        <is>
-          <t>session</t>
-        </is>
-      </c>
-      <c r="D27" s="34" t="n">
-        <v>28</v>
-      </c>
-      <c r="E27" s="35" t="n">
-        <v>43</v>
-      </c>
-      <c r="F27" s="36" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Déplacements &amp; terrain</t>
-        </is>
-      </c>
-      <c r="E28" s="44" t="n">
-        <v>16000</v>
-      </c>
-      <c r="F28" s="17" t="inlineStr">
-        <is>
-          <t>6.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="30" t="inlineStr">
-        <is>
-          <t>6. FORMATION ET ATELIERS</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="31" t="inlineStr">
-        <is>
-          <t>Formation des 14 coordinateurs locaux (protocoles, outils d'enregistrement)</t>
-        </is>
-      </c>
-      <c r="B30" s="32" t="inlineStr">
-        <is>
-          <t>Salle + matériel + indemnités — 2 jours</t>
-        </is>
-      </c>
-      <c r="C30" s="33" t="inlineStr">
-        <is>
-          <t>forfait</t>
-        </is>
-      </c>
-      <c r="D30" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="35" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F30" s="36" t="n">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="37" t="inlineStr">
-        <is>
-          <t>Atelier de restitution final — communauté NLP africaine</t>
-        </is>
-      </c>
-      <c r="B31" s="38" t="inlineStr">
-        <is>
-          <t>Organisation, accueil participants, matériel de présentation</t>
-        </is>
-      </c>
-      <c r="C31" s="39" t="inlineStr">
-        <is>
-          <t>forfait</t>
-        </is>
-      </c>
-      <c r="D31" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="41" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F31" s="42" t="n">
-        <v>2000</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="31" t="inlineStr">
         <is>
-          <t>Participation à une conférence NLP régionale (ex. IndabaX)</t>
+          <t>Missions régionales — avions intérieurs + taxi-brousse (14 régions, 2 visites)</t>
         </is>
       </c>
       <c r="B32" s="32" t="inlineStr">
         <is>
-          <t>Inscription + transport + hébergement</t>
+          <t>400 × 14 régions × 2 allers-retours</t>
         </is>
       </c>
       <c r="C32" s="33" t="inlineStr">
         <is>
+          <t>mission</t>
+        </is>
+      </c>
+      <c r="D32" s="34" t="n">
+        <v>28</v>
+      </c>
+      <c r="E32" s="35" t="n">
+        <v>400</v>
+      </c>
+      <c r="F32" s="36" t="n">
+        <v>11200</v>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="37" t="inlineStr">
+        <is>
+          <t>Per diem et hébergement — superviseurs terrain</t>
+        </is>
+      </c>
+      <c r="B33" s="38" t="inlineStr">
+        <is>
+          <t>50/j × 3 j × 14 régions × 2 visites</t>
+        </is>
+      </c>
+      <c r="C33" s="39" t="inlineStr">
+        <is>
+          <t>j×mission</t>
+        </is>
+      </c>
+      <c r="D33" s="40" t="n">
+        <v>84</v>
+      </c>
+      <c r="E33" s="41" t="n">
+        <v>50</v>
+      </c>
+      <c r="F33" s="42" t="n">
+        <v>4200</v>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="31" t="inlineStr">
+        <is>
+          <t>Location de salles communautaires pour les sessions de collecte</t>
+        </is>
+      </c>
+      <c r="B34" s="32" t="inlineStr">
+        <is>
+          <t>43 × 14 régions × 2 sessions  +  réserve imprévus</t>
+        </is>
+      </c>
+      <c r="C34" s="33" t="inlineStr">
+        <is>
+          <t>session</t>
+        </is>
+      </c>
+      <c r="D34" s="34" t="n">
+        <v>28</v>
+      </c>
+      <c r="E34" s="35" t="n">
+        <v>43</v>
+      </c>
+      <c r="F34" s="36" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Déplacements &amp; terrain</t>
+        </is>
+      </c>
+      <c r="E35" s="44" t="n">
+        <v>16000</v>
+      </c>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>6.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="30" t="inlineStr">
+        <is>
+          <t>6. FORMATION ET ATELIERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="31" t="inlineStr">
+        <is>
+          <t>Formation des 14 coordinateurs locaux (protocoles, outils d'enregistrement)</t>
+        </is>
+      </c>
+      <c r="B37" s="32" t="inlineStr">
+        <is>
+          <t>Salle + matériel + indemnités — 2 jours</t>
+        </is>
+      </c>
+      <c r="C37" s="33" t="inlineStr">
+        <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D32" s="34" t="n">
+      <c r="D37" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="35" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F32" s="36" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Formation &amp; ateliers</t>
-        </is>
-      </c>
-      <c r="E33" s="44" t="n">
-        <v>4500</v>
-      </c>
-      <c r="F33" s="17" t="inlineStr">
-        <is>
-          <t>1.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="30" t="inlineStr">
-        <is>
-          <t>7. COMMUNICATION ET DOCUMENTATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="31" t="inlineStr">
-        <is>
-          <t>Rapports d'avancement semestriels (mise en page, traduction FR/EN)</t>
-        </is>
-      </c>
-      <c r="B35" s="32" t="inlineStr">
-        <is>
-          <t>250 × 6 rapports (M3, M6, M9, M12, M15, M18)</t>
-        </is>
-      </c>
-      <c r="C35" s="33" t="inlineStr">
-        <is>
-          <t>rapport</t>
-        </is>
-      </c>
-      <c r="D35" s="34" t="n">
-        <v>6</v>
-      </c>
-      <c r="E35" s="35" t="n">
-        <v>100</v>
-      </c>
-      <c r="F35" s="36" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="37" t="inlineStr">
-        <is>
-          <t>Outils numériques : gestion projet, hébergement web, licences</t>
-        </is>
-      </c>
-      <c r="B36" s="38" t="inlineStr">
-        <is>
-          <t>50/mois × 18 mois</t>
-        </is>
-      </c>
-      <c r="C36" s="39" t="inlineStr">
-        <is>
-          <t>mois</t>
-        </is>
-      </c>
-      <c r="D36" s="40" t="n">
-        <v>18</v>
-      </c>
-      <c r="E36" s="41" t="n">
-        <v>50</v>
-      </c>
-      <c r="F36" s="42" t="n">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Communication</t>
-        </is>
-      </c>
-      <c r="E37" s="44" t="n">
+      <c r="E37" s="35" t="n">
         <v>1500</v>
       </c>
-      <c r="F37" s="17" t="inlineStr">
-        <is>
-          <t>0.6%</t>
-        </is>
+      <c r="F37" s="36" t="n">
+        <v>1500</v>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="30" t="inlineStr">
-        <is>
-          <t>8. AUTRES COÛTS DIRECTS</t>
-        </is>
+      <c r="A38" s="37" t="inlineStr">
+        <is>
+          <t>Atelier de restitution final — communauté NLP africaine</t>
+        </is>
+      </c>
+      <c r="B38" s="38" t="inlineStr">
+        <is>
+          <t>Organisation, accueil participants, matériel de présentation</t>
+        </is>
+      </c>
+      <c r="C38" s="39" t="inlineStr">
+        <is>
+          <t>forfait</t>
+        </is>
+      </c>
+      <c r="D38" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="41" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F38" s="42" t="n">
+        <v>2000</v>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="31" t="inlineStr">
         <is>
-          <t>Frais administratifs et juridiques (contrats, enregistrements officiels)</t>
+          <t>Participation à une conférence NLP régionale (ex. IndabaX)</t>
         </is>
       </c>
       <c r="B39" s="32" t="inlineStr">
         <is>
-          <t>Notaire, administration, légalisation</t>
+          <t>Inscription + transport + hébergement</t>
         </is>
       </c>
       <c r="C39" s="33" t="inlineStr">
@@ -1947,354 +2018,475 @@
         <v>1</v>
       </c>
       <c r="E39" s="35" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F39" s="36" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Formation &amp; ateliers</t>
+        </is>
+      </c>
+      <c r="E40" s="44" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F40" s="17" t="inlineStr">
+        <is>
+          <t>1.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>7. COMMUNICATION ET DOCUMENTATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="31" t="inlineStr">
+        <is>
+          <t>Rapports d'avancement semestriels (mise en page, traduction FR/EN)</t>
+        </is>
+      </c>
+      <c r="B42" s="32" t="inlineStr">
+        <is>
+          <t>250 × 6 rapports (M3, M6, M9, M12, M15, M18)</t>
+        </is>
+      </c>
+      <c r="C42" s="33" t="inlineStr">
+        <is>
+          <t>rapport</t>
+        </is>
+      </c>
+      <c r="D42" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E42" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="F42" s="36" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="37" t="inlineStr">
+        <is>
+          <t>Outils numériques : gestion projet, hébergement web, licences</t>
+        </is>
+      </c>
+      <c r="B43" s="38" t="inlineStr">
+        <is>
+          <t>50/mois × 18 mois</t>
+        </is>
+      </c>
+      <c r="C43" s="39" t="inlineStr">
+        <is>
+          <t>mois</t>
+        </is>
+      </c>
+      <c r="D43" s="40" t="n">
+        <v>18</v>
+      </c>
+      <c r="E43" s="41" t="n">
+        <v>50</v>
+      </c>
+      <c r="F43" s="42" t="n">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Communication</t>
+        </is>
+      </c>
+      <c r="E44" s="44" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F44" s="17" t="inlineStr">
+        <is>
+          <t>0.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="30" t="inlineStr">
+        <is>
+          <t>8. AUTRES COÛTS DIRECTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="31" t="inlineStr">
+        <is>
+          <t>Frais administratifs et juridiques (contrats, enregistrements officiels)</t>
+        </is>
+      </c>
+      <c r="B46" s="32" t="inlineStr">
+        <is>
+          <t>Notaire, administration, légalisation</t>
+        </is>
+      </c>
+      <c r="C46" s="33" t="inlineStr">
+        <is>
+          <t>forfait</t>
+        </is>
+      </c>
+      <c r="D46" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="35" t="n">
         <v>500</v>
       </c>
-      <c r="F39" s="36" t="n">
+      <c r="F46" s="36" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="37" t="inlineStr">
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="37" t="inlineStr">
         <is>
           <t>Réserve pour imprévus opérationnels</t>
         </is>
       </c>
-      <c r="B40" s="38" t="inlineStr">
+      <c r="B47" s="38" t="inlineStr">
         <is>
           <t>Ajustements terrain non anticipés</t>
         </is>
       </c>
-      <c r="C40" s="39" t="inlineStr">
+      <c r="C47" s="39" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D40" s="40" t="n">
+      <c r="D47" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E40" s="41" t="n">
+      <c r="E47" s="41" t="n">
         <v>500</v>
       </c>
-      <c r="F40" s="42" t="n">
+      <c r="F47" s="42" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="43" t="inlineStr">
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="43" t="inlineStr">
         <is>
           <t>Sous-total Autres coûts directs</t>
         </is>
       </c>
-      <c r="E41" s="44" t="n">
+      <c r="E48" s="44" t="n">
         <v>1000</v>
       </c>
-      <c r="F41" s="17" t="inlineStr">
+      <c r="F48" s="17" t="inlineStr">
         <is>
           <t>0.4%</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="24" customHeight="1">
-      <c r="A42" s="46" t="inlineStr">
+    <row r="49" ht="24" customHeight="1">
+      <c r="A49" s="45" t="inlineStr">
         <is>
           <t>TOTAL DES COÛTS DIRECTS</t>
         </is>
       </c>
-      <c r="E42" s="47" t="n">
-        <v>233428</v>
-      </c>
-      <c r="F42" s="48" t="inlineStr">
+      <c r="E49" s="46" t="n">
+        <v>238083</v>
+      </c>
+      <c r="F49" s="47" t="inlineStr">
         <is>
           <t>100 %</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="43" t="inlineStr">
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="43" t="inlineStr">
         <is>
           <t>Frais généraux / Coûts indirects (5 % des coûts directs)</t>
         </is>
       </c>
-      <c r="E43" s="44" t="n">
-        <v>11671</v>
-      </c>
-      <c r="F43" s="49" t="inlineStr">
-        <is>
-          <t>5 % × 233 428</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="28" customHeight="1">
-      <c r="A44" s="18" t="inlineStr">
+      <c r="E50" s="44" t="n">
+        <v>11904</v>
+      </c>
+      <c r="F50" s="48" t="inlineStr">
+        <is>
+          <t>5 % × 238 083</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="18" t="inlineStr">
         <is>
           <t>GRAND TOTAL — BUDGET CASH DEMANDÉ  (plafond Cat. 3 : 250 000 USD)</t>
         </is>
       </c>
-      <c r="E44" s="50" t="n">
-        <v>245099</v>
-      </c>
-      <c r="F44" s="51" t="inlineStr">
+      <c r="E51" s="49" t="n">
+        <v>249987</v>
+      </c>
+      <c r="F51" s="50" t="inlineStr">
         <is>
           <t>&lt; 250 000 USD ✓</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="52" t="inlineStr">
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="51" t="inlineStr">
         <is>
           <t>9. RESSOURCES DE CALCUL GCP — Q18  (crédits séparés du budget cash — plafond 400 000 USD)</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="31" t="inlineStr">
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="31" t="inlineStr">
         <is>
           <t>Vertex AI Custom Training — fine-tuning NLLB LoRA (6 langues × 18 dialectes)</t>
         </is>
       </c>
-      <c r="B47" s="32" t="inlineStr">
+      <c r="B54" s="32" t="inlineStr">
         <is>
           <t>L4 Spot ~0,28 $/h — expérimentations + runs finaux</t>
         </is>
       </c>
-      <c r="C47" s="33" t="inlineStr">
+      <c r="C54" s="33" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D47" s="34" t="n">
+      <c r="D54" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="E47" s="35" t="n">
+      <c r="E54" s="35" t="n">
         <v>45000</v>
       </c>
-      <c r="F47" s="36" t="n">
+      <c r="F54" s="36" t="n">
         <v>45000</v>
       </c>
     </row>
-    <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="37" t="inlineStr">
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="37" t="inlineStr">
         <is>
           <t>Vertex AI Custom Training — fine-tuning MMS-TTS VITS (18 dialectes)</t>
         </is>
       </c>
-      <c r="B48" s="38" t="inlineStr">
+      <c r="B55" s="38" t="inlineStr">
         <is>
           <t>18 dialectes × 3 cycles × 1,5 h GPU + hyperparamètres</t>
         </is>
       </c>
-      <c r="C48" s="39" t="inlineStr">
+      <c r="C55" s="39" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D48" s="40" t="n">
+      <c r="D55" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E48" s="41" t="n">
+      <c r="E55" s="41" t="n">
         <v>20000</v>
       </c>
-      <c r="F48" s="42" t="n">
+      <c r="F55" s="42" t="n">
         <v>20000</v>
       </c>
     </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="31" t="inlineStr">
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="31" t="inlineStr">
         <is>
           <t>Vertex AI Custom Training — buffer expérimentation &amp; réentraînement</t>
         </is>
       </c>
-      <c r="B49" s="32" t="inlineStr">
+      <c r="B56" s="32" t="inlineStr">
         <is>
           <t>Nouvelles données M10–M18, réentraînements itératifs</t>
         </is>
       </c>
-      <c r="C49" s="33" t="inlineStr">
+      <c r="C56" s="33" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D49" s="34" t="n">
+      <c r="D56" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="E49" s="35" t="n">
+      <c r="E56" s="35" t="n">
         <v>15000</v>
       </c>
-      <c r="F49" s="36" t="n">
+      <c r="F56" s="36" t="n">
         <v>15000</v>
       </c>
     </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="37" t="inlineStr">
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="37" t="inlineStr">
         <is>
           <t>Cloud Run GPU (NVIDIA L4 24 Go) — API MGVaovao en production</t>
         </is>
       </c>
-      <c r="B50" s="38" t="inlineStr">
+      <c r="B57" s="38" t="inlineStr">
         <is>
           <t>~2 500 $/mois × 18 mois — scale-to-zero hors heures</t>
         </is>
       </c>
-      <c r="C50" s="39" t="inlineStr">
+      <c r="C57" s="39" t="inlineStr">
         <is>
           <t>mois</t>
         </is>
       </c>
-      <c r="D50" s="40" t="n">
+      <c r="D57" s="40" t="n">
         <v>18</v>
       </c>
-      <c r="E50" s="41" t="n">
+      <c r="E57" s="41" t="n">
         <v>2500</v>
       </c>
-      <c r="F50" s="42" t="n">
+      <c r="F57" s="42" t="n">
         <v>45000</v>
       </c>
     </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="31" t="inlineStr">
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="31" t="inlineStr">
         <is>
           <t>GCS — stockage corpus audio + checkpoints (≈ 3 To)</t>
         </is>
       </c>
-      <c r="B51" s="32" t="inlineStr">
+      <c r="B58" s="32" t="inlineStr">
         <is>
           <t>0,02 $/Go/mois × 3 000 Go × 18 mois + egress</t>
         </is>
       </c>
-      <c r="C51" s="33" t="inlineStr">
+      <c r="C58" s="33" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D51" s="34" t="n">
+      <c r="D58" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="E51" s="35" t="n">
+      <c r="E58" s="35" t="n">
         <v>1500</v>
       </c>
-      <c r="F51" s="36" t="n">
+      <c r="F58" s="36" t="n">
         <v>1500</v>
       </c>
     </row>
-    <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="37" t="inlineStr">
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="37" t="inlineStr">
         <is>
           <t>Vertex AI Pipelines — orchestration MLOps Kubeflow DAG</t>
         </is>
       </c>
-      <c r="B52" s="38" t="inlineStr">
+      <c r="B59" s="38" t="inlineStr">
         <is>
           <t>0,03 $/run × ~500 runs + monitoring continu</t>
         </is>
       </c>
-      <c r="C52" s="39" t="inlineStr">
+      <c r="C59" s="39" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D52" s="40" t="n">
+      <c r="D59" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E52" s="41" t="n">
+      <c r="E59" s="41" t="n">
         <v>500</v>
       </c>
-      <c r="F52" s="42" t="n">
+      <c r="F59" s="42" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="31" t="inlineStr">
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="31" t="inlineStr">
         <is>
           <t>Cloud Build, Artifact Registry, Cloud Monitoring, Pub/Sub</t>
         </is>
       </c>
-      <c r="B53" s="32" t="inlineStr">
+      <c r="B60" s="32" t="inlineStr">
         <is>
           <t>CI/CD, registre d'images, alertes, déclencheurs GCS</t>
         </is>
       </c>
-      <c r="C53" s="33" t="inlineStr">
+      <c r="C60" s="33" t="inlineStr">
         <is>
           <t>mois</t>
         </is>
       </c>
-      <c r="D53" s="34" t="n">
+      <c r="D60" s="34" t="n">
         <v>18</v>
       </c>
-      <c r="E53" s="35" t="n">
+      <c r="E60" s="35" t="n">
         <v>139</v>
       </c>
-      <c r="F53" s="36" t="n">
+      <c r="F60" s="36" t="n">
         <v>2500</v>
       </c>
     </row>
-    <row r="54" ht="22" customHeight="1">
-      <c r="A54" s="37" t="inlineStr">
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="37" t="inlineStr">
         <is>
           <t>Dataflow / ingestion pipeline audio — traitement et normalisation</t>
         </is>
       </c>
-      <c r="B54" s="38" t="inlineStr">
+      <c r="B61" s="38" t="inlineStr">
         <is>
           <t>Ingestion et prétraitement audio en pipeline GCS</t>
         </is>
       </c>
-      <c r="C54" s="39" t="inlineStr">
+      <c r="C61" s="39" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D54" s="40" t="n">
+      <c r="D61" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E54" s="41" t="n">
+      <c r="E61" s="41" t="n">
         <v>20500</v>
       </c>
-      <c r="F54" s="42" t="n">
+      <c r="F61" s="42" t="n">
         <v>20500</v>
       </c>
     </row>
-    <row r="55" ht="28" customHeight="1">
-      <c r="A55" s="21" t="inlineStr">
+    <row r="62" ht="28" customHeight="1">
+      <c r="A62" s="21" t="inlineStr">
         <is>
           <t>TOTAL CRÉDITS GCP DEMANDÉS  (Q18b — séparé du budget cash)</t>
         </is>
       </c>
-      <c r="E55" s="53" t="n">
+      <c r="E62" s="52" t="n">
         <v>150000</v>
       </c>
-      <c r="F55" s="54" t="inlineStr">
+      <c r="F62" s="53" t="inlineStr">
         <is>
           <t>&lt; 400 000 USD ✓</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="24">
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A21:F21"/>
+  <mergeCells count="23">
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A62:D62"/>
     <mergeCell ref="A44:D44"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A24:D24"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A38:F38"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A41:D41"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A50:D50"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2316,229 +2508,229 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="55" t="inlineStr">
+      <c r="A1" s="54" t="inlineStr">
         <is>
           <t>RÉSUMÉ BUDGÉTAIRE — MGVaovao / LINGUA AFRICA 2026</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="56" t="inlineStr">
+      <c r="A2" s="55" t="inlineStr">
         <is>
           <t>Catégorie 3 — Applications sectorielles  |  Budget cash ≤ 250 000 USD  +  Crédits GCP ≤ 400 000 USD</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="57" t="inlineStr">
+      <c r="A3" s="56" t="inlineStr">
         <is>
           <t>Catégorie de coût</t>
         </is>
       </c>
-      <c r="B3" s="57" t="inlineStr">
+      <c r="B3" s="56" t="inlineStr">
         <is>
           <t>Montant (USD)</t>
         </is>
       </c>
-      <c r="C3" s="57" t="inlineStr">
+      <c r="C3" s="56" t="inlineStr">
         <is>
           <t>% coûts directs</t>
         </is>
       </c>
-      <c r="D3" s="57" t="inlineStr">
+      <c r="D3" s="56" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="58" t="inlineStr">
-        <is>
-          <t>1. Personnel — direction permanente</t>
-        </is>
-      </c>
-      <c r="B4" s="59" t="n">
-        <v>144900</v>
-      </c>
-      <c r="C4" s="60" t="inlineStr">
-        <is>
-          <t>62.1 %</t>
-        </is>
-      </c>
-      <c r="D4" s="60" t="inlineStr">
-        <is>
-          <t>5 postes : direction, ML, data ops, partenariats — 18 mois</t>
+      <c r="A4" s="57" t="inlineStr">
+        <is>
+          <t>1. Personnel — direction + équipe technique</t>
+        </is>
+      </c>
+      <c r="B4" s="58" t="n">
+        <v>192852</v>
+      </c>
+      <c r="C4" s="59" t="inlineStr">
+        <is>
+          <t>81.0 %</t>
+        </is>
+      </c>
+      <c r="D4" s="59" t="inlineStr">
+        <is>
+          <t>13 postes : 5 direction + 8 développeurs à 1 500 000 MGA/mois — 18 mois</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="61" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>2. Équipement et logiciels</t>
         </is>
       </c>
-      <c r="B5" s="62" t="n">
+      <c r="B5" s="61" t="n">
         <v>8000</v>
       </c>
-      <c r="C5" s="63" t="inlineStr">
+      <c r="C5" s="62" t="inlineStr">
         <is>
           <t xml:space="preserve"> 3.4 %</t>
         </is>
       </c>
-      <c r="D5" s="63" t="inlineStr">
+      <c r="D5" s="62" t="inlineStr">
         <is>
           <t>Laptops, matériel d'enregistrement terrain, connectivité</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="58" t="inlineStr">
+      <c r="A6" s="57" t="inlineStr">
         <is>
           <t>3. Collecte terrain</t>
         </is>
       </c>
-      <c r="B6" s="59" t="n">
-        <v>28728</v>
-      </c>
-      <c r="C6" s="60" t="inlineStr">
-        <is>
-          <t>12.3 %</t>
-        </is>
-      </c>
-      <c r="D6" s="60" t="inlineStr">
-        <is>
-          <t>54 collecteurs × 133 USD/mois × 4 mois — 3 par dialecte × 18</t>
+      <c r="B6" s="58" t="n">
+        <v>10640</v>
+      </c>
+      <c r="C6" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 4.5 %</t>
+        </is>
+      </c>
+      <c r="D6" s="59" t="inlineStr">
+        <is>
+          <t>20 collecteurs × 133 USD/mois × 4 mois</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="61" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>4. Annotation et ground truth</t>
         </is>
       </c>
-      <c r="B7" s="62" t="n">
-        <v>28800</v>
-      </c>
-      <c r="C7" s="63" t="inlineStr">
-        <is>
-          <t>12.3 %</t>
-        </is>
-      </c>
-      <c r="D7" s="63" t="inlineStr">
-        <is>
-          <t>36 annotateurs × 200 USD/mois × 4 mois — 2 par dialecte × 18</t>
+      <c r="B7" s="61" t="n">
+        <v>3591</v>
+      </c>
+      <c r="C7" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1.5 %</t>
+        </is>
+      </c>
+      <c r="D7" s="62" t="inlineStr">
+        <is>
+          <t>9 annotateurs × 133 USD/mois × 3 mois</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="58" t="inlineStr">
+      <c r="A8" s="57" t="inlineStr">
         <is>
           <t>5. Déplacements et terrain</t>
         </is>
       </c>
-      <c r="B8" s="59" t="n">
+      <c r="B8" s="58" t="n">
         <v>16000</v>
       </c>
-      <c r="C8" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6.9 %</t>
-        </is>
-      </c>
-      <c r="D8" s="60" t="inlineStr">
+      <c r="C8" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6.7 %</t>
+        </is>
+      </c>
+      <c r="D8" s="59" t="inlineStr">
         <is>
           <t>18 régions × 2 missions — avion, per diem, salles</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="61" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr">
         <is>
           <t>6. Formation et ateliers</t>
         </is>
       </c>
-      <c r="B9" s="62" t="n">
+      <c r="B9" s="61" t="n">
         <v>4500</v>
       </c>
-      <c r="C9" s="63" t="inlineStr">
+      <c r="C9" s="62" t="inlineStr">
         <is>
           <t xml:space="preserve"> 1.9 %</t>
         </is>
       </c>
-      <c r="D9" s="63" t="inlineStr">
+      <c r="D9" s="62" t="inlineStr">
         <is>
           <t>Formation équipes terrain + atelier restitution + conférence</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="58" t="inlineStr">
+      <c r="A10" s="57" t="inlineStr">
         <is>
           <t>7. Communication et documentation</t>
         </is>
       </c>
-      <c r="B10" s="59" t="n">
+      <c r="B10" s="58" t="n">
         <v>1500</v>
       </c>
-      <c r="C10" s="60" t="inlineStr">
+      <c r="C10" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve"> 0.6 %</t>
         </is>
       </c>
-      <c r="D10" s="60" t="inlineStr">
+      <c r="D10" s="59" t="inlineStr">
         <is>
           <t>Rapports semestriels, outils numériques</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="61" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr">
         <is>
           <t>8. Autres coûts directs</t>
         </is>
       </c>
-      <c r="B11" s="62" t="n">
+      <c r="B11" s="61" t="n">
         <v>1000</v>
       </c>
-      <c r="C11" s="63" t="inlineStr">
+      <c r="C11" s="62" t="inlineStr">
         <is>
           <t xml:space="preserve"> 0.4 %</t>
         </is>
       </c>
-      <c r="D11" s="63" t="inlineStr">
+      <c r="D11" s="62" t="inlineStr">
         <is>
           <t>Frais administratifs + réserve imprévus</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="64" t="inlineStr">
+      <c r="A12" s="63" t="inlineStr">
         <is>
           <t>TOTAL DES COÛTS DIRECTS</t>
         </is>
       </c>
-      <c r="B12" s="47" t="n">
-        <v>233428</v>
-      </c>
-      <c r="C12" s="48" t="inlineStr">
+      <c r="B12" s="46" t="n">
+        <v>238083</v>
+      </c>
+      <c r="C12" s="47" t="inlineStr">
         <is>
           <t>100 %</t>
         </is>
       </c>
-      <c r="D12" s="48" t="inlineStr">
-        <is>
-          <t>209 500 USD</t>
+      <c r="D12" s="47" t="inlineStr">
+        <is>
+          <t>238 083 USD</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="65" t="inlineStr">
+      <c r="A13" s="64" t="inlineStr">
         <is>
           <t>Frais généraux / indirects (5 %)</t>
         </is>
       </c>
       <c r="B13" s="44" t="n">
-        <v>11671</v>
+        <v>11904</v>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
@@ -2547,112 +2739,112 @@
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
-          <t>5 % × 233 428</t>
+          <t>5 % × 238 083</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="66" t="inlineStr">
+      <c r="A14" s="65" t="inlineStr">
         <is>
           <t>GRAND TOTAL — BUDGET CASH DEMANDÉ</t>
         </is>
       </c>
-      <c r="B14" s="50" t="n">
-        <v>245099</v>
-      </c>
-      <c r="C14" s="67" t="inlineStr">
+      <c r="B14" s="49" t="n">
+        <v>249987</v>
+      </c>
+      <c r="C14" s="66" t="inlineStr">
         <is>
           <t>&lt; 250 000 USD ✓</t>
         </is>
       </c>
-      <c r="D14" s="67" t="inlineStr">
+      <c r="D14" s="66" t="inlineStr">
         <is>
           <t>Plafond Cat. 3 respecté</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="68" t="inlineStr">
+      <c r="A16" s="67" t="inlineStr">
         <is>
           <t>RESSOURCES DE CALCUL GCP — Q18  (séparées du budget cash — plafond 400 000 USD)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="58" t="inlineStr">
+      <c r="A17" s="57" t="inlineStr">
         <is>
           <t>Vertex AI Custom Training — NLLB LoRA + MMS-TTS + expérimentation</t>
         </is>
       </c>
-      <c r="B17" s="59" t="n">
+      <c r="B17" s="58" t="n">
         <v>80000</v>
       </c>
-      <c r="C17" s="60" t="inlineStr">
+      <c r="C17" s="59" t="inlineStr">
         <is>
           <t>53.3 %</t>
         </is>
       </c>
-      <c r="D17" s="60" t="inlineStr">
+      <c r="D17" s="59" t="inlineStr">
         <is>
           <t>6 langues × 18 dialectes + cycles itératifs</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="61" t="inlineStr">
+      <c r="A18" s="60" t="inlineStr">
         <is>
           <t>Cloud Run GPU — infrastructure de production API (18 mois)</t>
         </is>
       </c>
-      <c r="B18" s="62" t="n">
+      <c r="B18" s="61" t="n">
         <v>45000</v>
       </c>
-      <c r="C18" s="63" t="inlineStr">
+      <c r="C18" s="62" t="inlineStr">
         <is>
           <t>30.0 %</t>
         </is>
       </c>
-      <c r="D18" s="63" t="inlineStr">
+      <c r="D18" s="62" t="inlineStr">
         <is>
           <t>NVIDIA L4 24 Go — scale-to-zero hors heures</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="58" t="inlineStr">
+      <c r="A19" s="57" t="inlineStr">
         <is>
           <t>GCS, Pipelines, CI/CD, Monitoring, Dataflow, Pub/Sub</t>
         </is>
       </c>
-      <c r="B19" s="59" t="n">
+      <c r="B19" s="58" t="n">
         <v>25000</v>
       </c>
-      <c r="C19" s="60" t="inlineStr">
+      <c r="C19" s="59" t="inlineStr">
         <is>
           <t>16.7 %</t>
         </is>
       </c>
-      <c r="D19" s="60" t="inlineStr">
+      <c r="D19" s="59" t="inlineStr">
         <is>
           <t>Stockage 3 To + orchestration MLOps + ingestion</t>
         </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="69" t="inlineStr">
+      <c r="A20" s="68" t="inlineStr">
         <is>
           <t>TOTAL CRÉDITS GCP DEMANDÉS (Q18b)</t>
         </is>
       </c>
-      <c r="B20" s="53" t="n">
+      <c r="B20" s="52" t="n">
         <v>150000</v>
       </c>
-      <c r="C20" s="70" t="inlineStr">
+      <c r="C20" s="69" t="inlineStr">
         <is>
           <t>&lt; 400 000 USD ✓</t>
         </is>
       </c>
-      <c r="D20" s="70" t="inlineStr">
+      <c r="D20" s="69" t="inlineStr">
         <is>
           <t>Plafond Q18 respecté</t>
         </is>

</xml_diff>

<commit_message>
Refactor budget: 12 postes, salaires ajustés, tour Madagascar, synchro Excel/DOCX
- Réduit salaires directrice et chefs de projet à 1 333 USD/mois (6 000 000 MGA)
- Supprime développeur full-stack, ajoute développeur mobile (12 postes au total)
- Supprime doublon développeur IA/ML engineer (un seul poste)
- Fusionne sections collecte et annotation → "Collecte et traitement des données" (14 231 USD)
- Augmente déplacements à 20 000 USD (transport local coordinateurs)
- Augmente formation/ateliers à 22 000 USD (tournée nationale 18 villes)
- Porte communication à 2 500 USD (stratégie réseaux sociaux)
- Nouveau total : 220 167 directs + 5 % frais généraux = 231 175 USD
- Synchronise Excel (generate_budget.py), DOCX FR et EN, LINGUA_Africa_Application_QA.md
- Supprime noms personnels dans Excel, titres de postes uniquement
- Ajoute référence docs privées dans .gitignore
</commit_message>
<xml_diff>
--- a/LINGUA_Africa_Budget_Detaille.xlsx
+++ b/LINGUA_Africa_Budget_Detaille.xlsx
@@ -891,15 +891,15 @@
       <c r="A9" s="1" t="inlineStr"/>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Personnel — direction + équipe technique (13 postes)</t>
+          <t>Personnel — direction + équipe technique (12 postes)</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>192852</v>
+        <v>152436</v>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>81.0 % des coûts directs</t>
+          <t>69.2 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -915,7 +915,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 3.4 % des coûts directs</t>
+          <t xml:space="preserve"> 3.6 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -923,15 +923,15 @@
       <c r="A11" s="1" t="inlineStr"/>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Collecte terrain (20 collecteurs)</t>
+          <t>Collecte et traitement des données (20 collecteurs + 9 annotateurs)</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>10640</v>
+        <v>14231</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 4.5 % des coûts directs</t>
+          <t xml:space="preserve"> 6.5 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -939,15 +939,15 @@
       <c r="A12" s="1" t="inlineStr"/>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Annotation ground truth (9 annotateurs)</t>
+          <t>Déplacements et terrain (tournée 14 régions)</t>
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>3591</v>
+        <v>20000</v>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 1.5 % des coûts directs</t>
+          <t xml:space="preserve"> 9.1 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -955,15 +955,15 @@
       <c r="A13" s="1" t="inlineStr"/>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Déplacements et terrain</t>
+          <t>Formation et ateliers (tournée nationale 18 villes)</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>16000</v>
+        <v>22000</v>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 6.7 % des coûts directs</t>
+          <t>10.0 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -971,15 +971,15 @@
       <c r="A14" s="1" t="inlineStr"/>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Formation et ateliers</t>
+          <t>Communication et mobilisation</t>
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>4500</v>
+        <v>2500</v>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 1.9 % des coûts directs</t>
+          <t xml:space="preserve"> 1.1 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -987,15 +987,15 @@
       <c r="A15" s="1" t="inlineStr"/>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Communication et autres coûts</t>
+          <t>Autres coûts directs</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 1.1 % des coûts directs</t>
+          <t xml:space="preserve"> 0.5 % des coûts directs</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>238083</v>
+        <v>220167</v>
       </c>
       <c r="D16" s="14" t="n"/>
     </row>
@@ -1022,11 +1022,11 @@
         </is>
       </c>
       <c r="C18" s="16" t="n">
-        <v>11904</v>
+        <v>11008</v>
       </c>
       <c r="D18" s="17" t="inlineStr">
         <is>
-          <t>5 % × 238 083</t>
+          <t>5 % × 220 167</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
         </is>
       </c>
       <c r="C19" s="19" t="n">
-        <v>249987</v>
+        <v>231175</v>
       </c>
       <c r="D19" s="20" t="inlineStr">
         <is>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C23" s="26" t="inlineStr">
         <is>
-          <t>github.com/mgvaovao/ml  |  github.com/mgvaovao/backend_ia</t>
+          <t>github.com/mgvaovao-Mdn/ml  |  github.com/mgvaovao-Mdn/backend_ia</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1267,7 +1267,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="31" t="inlineStr">
         <is>
-          <t>Fenitra Ravelomanantsoa — Fondateur, conseil stratégique (50 %)</t>
+          <t>Fondateur et Directeur général — conseil stratégique (50 %)</t>
         </is>
       </c>
       <c r="B5" s="32" t="inlineStr">
@@ -1293,12 +1293,12 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="37" t="inlineStr">
         <is>
-          <t>Norolala Randrianarison (Mme Noro) — Directrice locale (100 %)</t>
+          <t>Directrice locale (100 %)</t>
         </is>
       </c>
       <c r="B6" s="38" t="inlineStr">
         <is>
-          <t>2 000 × 18 mois</t>
+          <t>1 333 × 18 mois  ≈ 6 000 000 MGA/mois</t>
         </is>
       </c>
       <c r="C6" s="39" t="inlineStr">
@@ -1310,21 +1310,21 @@
         <v>18</v>
       </c>
       <c r="E6" s="41" t="n">
-        <v>2000</v>
+        <v>1333</v>
       </c>
       <c r="F6" s="42" t="n">
-        <v>36000</v>
+        <v>23994</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="31" t="inlineStr">
         <is>
-          <t>Guillaume Rakotonjanahary — Chef de projet technique ML/Dev (100 %)</t>
+          <t>Chef de projet technique ML/Dev (100 %)</t>
         </is>
       </c>
       <c r="B7" s="32" t="inlineStr">
         <is>
-          <t>1 800 × 18 mois</t>
+          <t>1 333 × 18 mois  ≈ 6 000 000 MGA/mois</t>
         </is>
       </c>
       <c r="C7" s="33" t="inlineStr">
@@ -1336,21 +1336,21 @@
         <v>18</v>
       </c>
       <c r="E7" s="35" t="n">
-        <v>1800</v>
+        <v>1333</v>
       </c>
       <c r="F7" s="36" t="n">
-        <v>32400</v>
+        <v>23994</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="37" t="inlineStr">
         <is>
-          <t>Karine Rajaofera — Chef de projet Data, Opérations &amp; Fonctionnel (100 %)</t>
+          <t>Chef de projet Data et Opérations (100 %)</t>
         </is>
       </c>
       <c r="B8" s="38" t="inlineStr">
         <is>
-          <t>1 800 × 18 mois</t>
+          <t>1 333 × 18 mois  ≈ 6 000 000 MGA/mois</t>
         </is>
       </c>
       <c r="C8" s="39" t="inlineStr">
@@ -1362,21 +1362,21 @@
         <v>18</v>
       </c>
       <c r="E8" s="41" t="n">
-        <v>1800</v>
+        <v>1333</v>
       </c>
       <c r="F8" s="42" t="n">
-        <v>32400</v>
+        <v>23994</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="31" t="inlineStr">
         <is>
-          <t>Chef de projet 3 — Partenariats &amp; impact (recrutement M7, 100 %)</t>
+          <t>Chef de projet Partenariats et Impact (recrutement M7, 100 %)</t>
         </is>
       </c>
       <c r="B9" s="32" t="inlineStr">
         <is>
-          <t>1 800 × 12 mois (M7–M18)</t>
+          <t>1 333 × 12 mois (M7–M18)  ≈ 6 000 000 MGA/mois</t>
         </is>
       </c>
       <c r="C9" s="33" t="inlineStr">
@@ -1388,10 +1388,10 @@
         <v>12</v>
       </c>
       <c r="E9" s="35" t="n">
-        <v>1800</v>
+        <v>1333</v>
       </c>
       <c r="F9" s="36" t="n">
-        <v>21600</v>
+        <v>15996</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -1449,7 +1449,7 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="37" t="inlineStr">
         <is>
-          <t>Développeur IA / ML engineer 1 (100 %)</t>
+          <t>Développeur mobile (100 %)</t>
         </is>
       </c>
       <c r="B12" s="38" t="inlineStr">
@@ -1475,7 +1475,7 @@
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="31" t="inlineStr">
         <is>
-          <t>Développeur IA / ML engineer 2 (100 %)</t>
+          <t>Développeur IA / ML engineer (100 %)</t>
         </is>
       </c>
       <c r="B13" s="32" t="inlineStr">
@@ -1501,7 +1501,7 @@
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="37" t="inlineStr">
         <is>
-          <t>Data scientist / ML engineer (100 %)</t>
+          <t>Data scientist (100 %)</t>
         </is>
       </c>
       <c r="B14" s="38" t="inlineStr">
@@ -1553,7 +1553,7 @@
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="37" t="inlineStr">
         <is>
-          <t>Développeur full-stack (100 %)</t>
+          <t>Data engineer (100 %)</t>
         </is>
       </c>
       <c r="B16" s="38" t="inlineStr">
@@ -1576,559 +1576,619 @@
         <v>5994</v>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="31" t="inlineStr">
-        <is>
-          <t>Data engineer (100 %)</t>
-        </is>
-      </c>
-      <c r="B17" s="32" t="inlineStr">
-        <is>
-          <t>333 × 18 mois  ≈ 1 500 000 MGA/mois</t>
-        </is>
-      </c>
-      <c r="C17" s="33" t="inlineStr">
-        <is>
-          <t>mois</t>
-        </is>
-      </c>
-      <c r="D17" s="34" t="n">
-        <v>18</v>
-      </c>
-      <c r="E17" s="35" t="n">
-        <v>333</v>
-      </c>
-      <c r="F17" s="36" t="n">
-        <v>5994</v>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="43" t="inlineStr">
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="43" t="inlineStr">
         <is>
           <t>Sous-total Personnel (direction + équipe technique)</t>
         </is>
       </c>
-      <c r="E18" s="44" t="n">
-        <v>192852</v>
-      </c>
-      <c r="F18" s="17" t="inlineStr">
-        <is>
-          <t>81.0%</t>
+      <c r="E17" s="44" t="n">
+        <v>152436</v>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>69.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>2. ÉQUIPEMENT ET LOGICIELS</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="30" t="inlineStr">
-        <is>
-          <t>2. ÉQUIPEMENT ET LOGICIELS</t>
-        </is>
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>Ordinateurs portables — équipe technique locale (hors fondateur à Zurich)</t>
+        </is>
+      </c>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>778 USD × 6 unités  (≈ 3 500 000 MGA l'unité)</t>
+        </is>
+      </c>
+      <c r="C19" s="33" t="inlineStr">
+        <is>
+          <t>unité</t>
+        </is>
+      </c>
+      <c r="D19" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E19" s="35" t="n">
+        <v>778</v>
+      </c>
+      <c r="F19" s="36" t="n">
+        <v>4667</v>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="31" t="inlineStr">
-        <is>
-          <t>Ordinateurs portables — équipe technique locale (hors fondateur à Zurich)</t>
-        </is>
-      </c>
-      <c r="B20" s="32" t="inlineStr">
-        <is>
-          <t>778 USD × 6 unités  (≈ 3 500 000 MGA l'unité)</t>
-        </is>
-      </c>
-      <c r="C20" s="33" t="inlineStr">
+      <c r="A20" s="37" t="inlineStr">
+        <is>
+          <t>Tablettes de terrain pour coordinateurs de collecte</t>
+        </is>
+      </c>
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t>150 × 14 coordinateurs</t>
+        </is>
+      </c>
+      <c r="C20" s="39" t="inlineStr">
         <is>
           <t>unité</t>
         </is>
       </c>
-      <c r="D20" s="34" t="n">
-        <v>6</v>
-      </c>
-      <c r="E20" s="35" t="n">
-        <v>778</v>
-      </c>
-      <c r="F20" s="36" t="n">
-        <v>4667</v>
+      <c r="D20" s="40" t="n">
+        <v>14</v>
+      </c>
+      <c r="E20" s="41" t="n">
+        <v>150</v>
+      </c>
+      <c r="F20" s="42" t="n">
+        <v>2100</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="37" t="inlineStr">
-        <is>
-          <t>Tablettes de terrain pour coordinateurs de collecte</t>
-        </is>
-      </c>
-      <c r="B21" s="38" t="inlineStr">
-        <is>
-          <t>150 × 14 coordinateurs</t>
-        </is>
-      </c>
-      <c r="C21" s="39" t="inlineStr">
+      <c r="A21" s="31" t="inlineStr">
+        <is>
+          <t>Microphones USB qualité ASR/TTS pour les sessions de collecte</t>
+        </is>
+      </c>
+      <c r="B21" s="32" t="inlineStr">
+        <is>
+          <t>50 × 14 coordinateurs</t>
+        </is>
+      </c>
+      <c r="C21" s="33" t="inlineStr">
         <is>
           <t>unité</t>
         </is>
       </c>
-      <c r="D21" s="40" t="n">
+      <c r="D21" s="34" t="n">
         <v>14</v>
       </c>
-      <c r="E21" s="41" t="n">
-        <v>150</v>
-      </c>
-      <c r="F21" s="42" t="n">
-        <v>2100</v>
+      <c r="E21" s="35" t="n">
+        <v>50</v>
+      </c>
+      <c r="F21" s="36" t="n">
+        <v>700</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="31" t="inlineStr">
-        <is>
-          <t>Microphones USB qualité ASR/TTS pour les sessions de collecte</t>
-        </is>
-      </c>
-      <c r="B22" s="32" t="inlineStr">
-        <is>
-          <t>50 × 14 coordinateurs</t>
-        </is>
-      </c>
-      <c r="C22" s="33" t="inlineStr">
-        <is>
-          <t>unité</t>
-        </is>
-      </c>
-      <c r="D22" s="34" t="n">
-        <v>14</v>
-      </c>
-      <c r="E22" s="35" t="n">
-        <v>50</v>
-      </c>
-      <c r="F22" s="36" t="n">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="37" t="inlineStr">
+      <c r="A22" s="37" t="inlineStr">
         <is>
           <t>Matériel de connectivité (routeurs Wi-Fi, dongles 4G régions rurales)</t>
         </is>
       </c>
-      <c r="B23" s="38" t="inlineStr">
+      <c r="B22" s="38" t="inlineStr">
         <is>
           <t>Forfait — 14 régions à faible infrastructure</t>
         </is>
       </c>
-      <c r="C23" s="39" t="inlineStr">
+      <c r="C22" s="39" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D23" s="40" t="n">
+      <c r="D22" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="41" t="n">
+      <c r="E22" s="41" t="n">
         <v>533</v>
       </c>
-      <c r="F23" s="42" t="n">
+      <c r="F22" s="42" t="n">
         <v>533</v>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="43" t="inlineStr">
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="43" t="inlineStr">
         <is>
           <t>Sous-total Équipement et logiciels</t>
         </is>
       </c>
-      <c r="E24" s="44" t="n">
+      <c r="E23" s="44" t="n">
         <v>8000</v>
       </c>
-      <c r="F24" s="17" t="inlineStr">
-        <is>
-          <t>3.4%</t>
+      <c r="F23" s="17" t="inlineStr">
+        <is>
+          <t>3.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>3. COLLECTE ET TRAITEMENT DES DONNÉES</t>
         </is>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="30" t="inlineStr">
-        <is>
-          <t>3. COLLECTE ET TRAITEMENT DE DONNÉES</t>
-        </is>
+      <c r="A25" s="31" t="inlineStr">
+        <is>
+          <t>20 collecteurs terrain — 1 à 2 par dialecte × 18 dialectes (recrutés dans les communautés, priorité aux femmes, rémunération équitable)</t>
+        </is>
+      </c>
+      <c r="B25" s="32" t="inlineStr">
+        <is>
+          <t>133 USD (600 000 MGA) × 20 pers. × 4 mois actifs</t>
+        </is>
+      </c>
+      <c r="C25" s="33" t="inlineStr">
+        <is>
+          <t>pers.×mois</t>
+        </is>
+      </c>
+      <c r="D25" s="34" t="n">
+        <v>80</v>
+      </c>
+      <c r="E25" s="35" t="n">
+        <v>133</v>
+      </c>
+      <c r="F25" s="36" t="n">
+        <v>10640</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="31" t="inlineStr">
-        <is>
-          <t>20 collecteurs terrain — 1 à 2 par dialecte × 18 dialectes (recrutés dans les communautés, priorité aux femmes, rémunération équitable)</t>
-        </is>
-      </c>
-      <c r="B26" s="32" t="inlineStr">
-        <is>
-          <t>133 USD (600 000 MGA) × 20 pers. × 4 mois actifs</t>
-        </is>
-      </c>
-      <c r="C26" s="33" t="inlineStr">
+      <c r="A26" s="37" t="inlineStr">
+        <is>
+          <t>9 annotateurs-transcripteurs — vérification des transcriptions, alignement phonème-graphème, contrôle qualité</t>
+        </is>
+      </c>
+      <c r="B26" s="38" t="inlineStr">
+        <is>
+          <t>133 USD (600 000 MGA) × 9 pers. × 3 mois actifs</t>
+        </is>
+      </c>
+      <c r="C26" s="39" t="inlineStr">
         <is>
           <t>pers.×mois</t>
         </is>
       </c>
-      <c r="D26" s="34" t="n">
-        <v>80</v>
-      </c>
-      <c r="E26" s="35" t="n">
+      <c r="D26" s="40" t="n">
+        <v>27</v>
+      </c>
+      <c r="E26" s="41" t="n">
         <v>133</v>
       </c>
-      <c r="F26" s="36" t="n">
-        <v>10640</v>
+      <c r="F26" s="42" t="n">
+        <v>3591</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="43" t="inlineStr">
         <is>
-          <t>Sous-total Collecte terrain</t>
+          <t>Sous-total Collecte et traitement des données</t>
         </is>
       </c>
       <c r="E27" s="44" t="n">
-        <v>10640</v>
+        <v>14231</v>
       </c>
       <c r="F27" s="17" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>6.5%</t>
         </is>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="30" t="inlineStr">
         <is>
-          <t>4. ANNOTATION ET VÉRIFICATION (GROUND TRUTH)</t>
+          <t>4. DÉPLACEMENTS ET TERRAIN</t>
         </is>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="31" t="inlineStr">
         <is>
-          <t>9 annotateurs-transcripteurs — vérification des transcriptions, alignement phonème-graphème, contrôle qualité</t>
+          <t>Missions régionales — avions intérieurs et taxi-brousse (14 régions, 2 visites par région)</t>
         </is>
       </c>
       <c r="B29" s="32" t="inlineStr">
         <is>
-          <t>133 USD (600 000 MGA) × 9 pers. × 3 mois actifs</t>
+          <t>400 × 14 régions × 2 allers-retours</t>
         </is>
       </c>
       <c r="C29" s="33" t="inlineStr">
         <is>
+          <t>mission</t>
+        </is>
+      </c>
+      <c r="D29" s="34" t="n">
+        <v>28</v>
+      </c>
+      <c r="E29" s="35" t="n">
+        <v>400</v>
+      </c>
+      <c r="F29" s="36" t="n">
+        <v>11200</v>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="37" t="inlineStr">
+        <is>
+          <t>Per diem et hébergement — superviseurs terrain</t>
+        </is>
+      </c>
+      <c r="B30" s="38" t="inlineStr">
+        <is>
+          <t>50/j × 3 j × 14 régions × 2 visites</t>
+        </is>
+      </c>
+      <c r="C30" s="39" t="inlineStr">
+        <is>
+          <t>j×mission</t>
+        </is>
+      </c>
+      <c r="D30" s="40" t="n">
+        <v>84</v>
+      </c>
+      <c r="E30" s="41" t="n">
+        <v>50</v>
+      </c>
+      <c r="F30" s="42" t="n">
+        <v>4200</v>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="31" t="inlineStr">
+        <is>
+          <t>Transport local pour les coordinateurs de collecte (déplacements intracommunautaires)</t>
+        </is>
+      </c>
+      <c r="B31" s="32" t="inlineStr">
+        <is>
+          <t>50 USD × 20 coordinateurs × 4 mois actifs</t>
+        </is>
+      </c>
+      <c r="C31" s="33" t="inlineStr">
+        <is>
           <t>pers.×mois</t>
         </is>
       </c>
-      <c r="D29" s="34" t="n">
-        <v>27</v>
-      </c>
-      <c r="E29" s="35" t="n">
-        <v>133</v>
-      </c>
-      <c r="F29" s="36" t="n">
-        <v>3591</v>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Annotation et ground truth</t>
-        </is>
-      </c>
-      <c r="E30" s="44" t="n">
-        <v>3591</v>
-      </c>
-      <c r="F30" s="17" t="inlineStr">
-        <is>
-          <t>1.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="30" t="inlineStr">
-        <is>
-          <t>5. DÉPLACEMENTS ET TERRAIN</t>
-        </is>
+      <c r="D31" s="34" t="n">
+        <v>80</v>
+      </c>
+      <c r="E31" s="35" t="n">
+        <v>50</v>
+      </c>
+      <c r="F31" s="36" t="n">
+        <v>4000</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="31" t="inlineStr">
-        <is>
-          <t>Missions régionales — avions intérieurs + taxi-brousse (14 régions, 2 visites)</t>
-        </is>
-      </c>
-      <c r="B32" s="32" t="inlineStr">
-        <is>
-          <t>400 × 14 régions × 2 allers-retours</t>
-        </is>
-      </c>
-      <c r="C32" s="33" t="inlineStr">
-        <is>
-          <t>mission</t>
-        </is>
-      </c>
-      <c r="D32" s="34" t="n">
+      <c r="A32" s="37" t="inlineStr">
+        <is>
+          <t>Location de salles communautaires pour les sessions de collecte et réserve imprévus</t>
+        </is>
+      </c>
+      <c r="B32" s="38" t="inlineStr">
+        <is>
+          <t>21 USD × 28 sessions + réserve opérationnelle</t>
+        </is>
+      </c>
+      <c r="C32" s="39" t="inlineStr">
+        <is>
+          <t>session</t>
+        </is>
+      </c>
+      <c r="D32" s="40" t="n">
         <v>28</v>
       </c>
-      <c r="E32" s="35" t="n">
-        <v>400</v>
-      </c>
-      <c r="F32" s="36" t="n">
-        <v>11200</v>
-      </c>
-    </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="37" t="inlineStr">
-        <is>
-          <t>Per diem et hébergement — superviseurs terrain</t>
-        </is>
-      </c>
-      <c r="B33" s="38" t="inlineStr">
-        <is>
-          <t>50/j × 3 j × 14 régions × 2 visites</t>
-        </is>
-      </c>
-      <c r="C33" s="39" t="inlineStr">
-        <is>
-          <t>j×mission</t>
-        </is>
-      </c>
-      <c r="D33" s="40" t="n">
-        <v>84</v>
-      </c>
-      <c r="E33" s="41" t="n">
-        <v>50</v>
-      </c>
-      <c r="F33" s="42" t="n">
-        <v>4200</v>
+      <c r="E32" s="41" t="n">
+        <v>21</v>
+      </c>
+      <c r="F32" s="42" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Déplacements et terrain</t>
+        </is>
+      </c>
+      <c r="E33" s="44" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F33" s="17" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="31" t="inlineStr">
-        <is>
-          <t>Location de salles communautaires pour les sessions de collecte</t>
-        </is>
-      </c>
-      <c r="B34" s="32" t="inlineStr">
-        <is>
-          <t>43 × 14 régions × 2 sessions  +  réserve imprévus</t>
-        </is>
-      </c>
-      <c r="C34" s="33" t="inlineStr">
-        <is>
-          <t>session</t>
-        </is>
-      </c>
-      <c r="D34" s="34" t="n">
-        <v>28</v>
-      </c>
-      <c r="E34" s="35" t="n">
-        <v>43</v>
-      </c>
-      <c r="F34" s="36" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Déplacements &amp; terrain</t>
-        </is>
-      </c>
-      <c r="E35" s="44" t="n">
-        <v>16000</v>
-      </c>
-      <c r="F35" s="17" t="inlineStr">
-        <is>
-          <t>6.7%</t>
-        </is>
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>5. FORMATION ET ATELIERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="31" t="inlineStr">
+        <is>
+          <t>Formation des coordinateurs locaux — protocoles, outils d'enregistrement (Antananarivo)</t>
+        </is>
+      </c>
+      <c r="B35" s="32" t="inlineStr">
+        <is>
+          <t>Salle + matériel + indemnités — 2 jours</t>
+        </is>
+      </c>
+      <c r="C35" s="33" t="inlineStr">
+        <is>
+          <t>forfait</t>
+        </is>
+      </c>
+      <c r="D35" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="35" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F35" s="36" t="n">
+        <v>1500</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="30" t="inlineStr">
-        <is>
-          <t>6. FORMATION ET ATELIERS</t>
-        </is>
+      <c r="A36" s="37" t="inlineStr">
+        <is>
+          <t>Tournée nationale de formation — 18 villes : transport intercity (avion et taxi-brousse)</t>
+        </is>
+      </c>
+      <c r="B36" s="38" t="inlineStr">
+        <is>
+          <t>300 USD × 18 étapes</t>
+        </is>
+      </c>
+      <c r="C36" s="39" t="inlineStr">
+        <is>
+          <t>étape</t>
+        </is>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>18</v>
+      </c>
+      <c r="E36" s="41" t="n">
+        <v>300</v>
+      </c>
+      <c r="F36" s="42" t="n">
+        <v>5400</v>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="31" t="inlineStr">
         <is>
-          <t>Formation des 14 coordinateurs locaux (protocoles, outils d'enregistrement)</t>
+          <t>Tournée nationale — hébergement équipe (18 villes × 3 nuits en moyenne)</t>
         </is>
       </c>
       <c r="B37" s="32" t="inlineStr">
         <is>
-          <t>Salle + matériel + indemnités — 2 jours</t>
+          <t>50 USD/nuit × 18 villes × 3 nuits</t>
         </is>
       </c>
       <c r="C37" s="33" t="inlineStr">
         <is>
-          <t>forfait</t>
+          <t>nuit</t>
         </is>
       </c>
       <c r="D37" s="34" t="n">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="E37" s="35" t="n">
-        <v>1500</v>
+        <v>50</v>
       </c>
       <c r="F37" s="36" t="n">
-        <v>1500</v>
+        <v>2700</v>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="37" t="inlineStr">
         <is>
-          <t>Atelier de restitution final — communauté NLP africaine</t>
+          <t>Tournée nationale — location de salles de conférence (18 villes)</t>
         </is>
       </c>
       <c r="B38" s="38" t="inlineStr">
         <is>
-          <t>Organisation, accueil participants, matériel de présentation</t>
+          <t>200 USD × 18 salles</t>
         </is>
       </c>
       <c r="C38" s="39" t="inlineStr">
         <is>
-          <t>forfait</t>
+          <t>salle</t>
         </is>
       </c>
       <c r="D38" s="40" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="E38" s="41" t="n">
-        <v>2000</v>
+        <v>200</v>
       </c>
       <c r="F38" s="42" t="n">
-        <v>2000</v>
+        <v>3600</v>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="31" t="inlineStr">
         <is>
-          <t>Participation à une conférence NLP régionale (ex. IndabaX)</t>
+          <t>Tournée nationale — matériel et supports pédagogiques (18 ateliers)</t>
         </is>
       </c>
       <c r="B39" s="32" t="inlineStr">
         <is>
+          <t>128 USD × 18 ateliers</t>
+        </is>
+      </c>
+      <c r="C39" s="33" t="inlineStr">
+        <is>
+          <t>atelier</t>
+        </is>
+      </c>
+      <c r="D39" s="34" t="n">
+        <v>18</v>
+      </c>
+      <c r="E39" s="35" t="n">
+        <v>128</v>
+      </c>
+      <c r="F39" s="36" t="n">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="37" t="inlineStr">
+        <is>
+          <t>Atelier de restitution final — communauté NLP africaine (Antananarivo)</t>
+        </is>
+      </c>
+      <c r="B40" s="38" t="inlineStr">
+        <is>
+          <t>Organisation, accueil participants, matériel de présentation</t>
+        </is>
+      </c>
+      <c r="C40" s="39" t="inlineStr">
+        <is>
+          <t>forfait</t>
+        </is>
+      </c>
+      <c r="D40" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="41" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F40" s="42" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="31" t="inlineStr">
+        <is>
+          <t>Participation à une conférence NLP régionale (IndabaX ou AfricaNLP)</t>
+        </is>
+      </c>
+      <c r="B41" s="32" t="inlineStr">
+        <is>
           <t>Inscription + transport + hébergement</t>
         </is>
       </c>
-      <c r="C39" s="33" t="inlineStr">
+      <c r="C41" s="33" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D39" s="34" t="n">
+      <c r="D41" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="E39" s="35" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F39" s="36" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Formation &amp; ateliers</t>
-        </is>
-      </c>
-      <c r="E40" s="44" t="n">
-        <v>4500</v>
-      </c>
-      <c r="F40" s="17" t="inlineStr">
-        <is>
-          <t>1.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="30" t="inlineStr">
-        <is>
-          <t>7. COMMUNICATION ET DOCUMENTATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="31" t="inlineStr">
+      <c r="E41" s="35" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F41" s="36" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Formation et ateliers</t>
+        </is>
+      </c>
+      <c r="E42" s="44" t="n">
+        <v>22000</v>
+      </c>
+      <c r="F42" s="17" t="inlineStr">
+        <is>
+          <t>10.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="30" t="inlineStr">
+        <is>
+          <t>6. COMMUNICATION ET MOBILISATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="31" t="inlineStr">
         <is>
           <t>Rapports d'avancement semestriels (mise en page, traduction FR/EN)</t>
         </is>
       </c>
-      <c r="B42" s="32" t="inlineStr">
-        <is>
-          <t>250 × 6 rapports (M3, M6, M9, M12, M15, M18)</t>
-        </is>
-      </c>
-      <c r="C42" s="33" t="inlineStr">
+      <c r="B44" s="32" t="inlineStr">
+        <is>
+          <t>100 × 6 rapports (M3, M6, M9, M12, M15, M18)</t>
+        </is>
+      </c>
+      <c r="C44" s="33" t="inlineStr">
         <is>
           <t>rapport</t>
         </is>
       </c>
-      <c r="D42" s="34" t="n">
+      <c r="D44" s="34" t="n">
         <v>6</v>
       </c>
-      <c r="E42" s="35" t="n">
+      <c r="E44" s="35" t="n">
         <v>100</v>
       </c>
-      <c r="F42" s="36" t="n">
+      <c r="F44" s="36" t="n">
         <v>600</v>
       </c>
     </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="37" t="inlineStr">
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="37" t="inlineStr">
         <is>
           <t>Outils numériques : gestion projet, hébergement web, licences</t>
         </is>
       </c>
-      <c r="B43" s="38" t="inlineStr">
+      <c r="B45" s="38" t="inlineStr">
         <is>
           <t>50/mois × 18 mois</t>
         </is>
       </c>
-      <c r="C43" s="39" t="inlineStr">
+      <c r="C45" s="39" t="inlineStr">
         <is>
           <t>mois</t>
         </is>
       </c>
-      <c r="D43" s="40" t="n">
+      <c r="D45" s="40" t="n">
         <v>18</v>
       </c>
-      <c r="E43" s="41" t="n">
+      <c r="E45" s="41" t="n">
         <v>50</v>
       </c>
-      <c r="F43" s="42" t="n">
+      <c r="F45" s="42" t="n">
         <v>900</v>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="43" t="inlineStr">
-        <is>
-          <t>Sous-total Communication</t>
-        </is>
-      </c>
-      <c r="E44" s="44" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F44" s="17" t="inlineStr">
-        <is>
-          <t>0.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="30" t="inlineStr">
-        <is>
-          <t>8. AUTRES COÛTS DIRECTS</t>
-        </is>
       </c>
     </row>
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="31" t="inlineStr">
         <is>
-          <t>Frais administratifs et juridiques (contrats, enregistrements officiels)</t>
+          <t>Stratégie de communication et réseaux sociaux (identité visuelle, contenus numériques)</t>
         </is>
       </c>
       <c r="B46" s="32" t="inlineStr">
         <is>
-          <t>Notaire, administration, légalisation</t>
+          <t>Forfait production contenus + community management</t>
         </is>
       </c>
       <c r="C46" s="33" t="inlineStr">
@@ -2140,353 +2200,399 @@
         <v>1</v>
       </c>
       <c r="E46" s="35" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F46" s="36" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="43" t="inlineStr">
+        <is>
+          <t>Sous-total Communication et mobilisation</t>
+        </is>
+      </c>
+      <c r="E47" s="44" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F47" s="17" t="inlineStr">
+        <is>
+          <t>1.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="30" t="inlineStr">
+        <is>
+          <t>7. AUTRES COÛTS DIRECTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="31" t="inlineStr">
+        <is>
+          <t>Frais administratifs et juridiques (contrats, enregistrements officiels)</t>
+        </is>
+      </c>
+      <c r="B49" s="32" t="inlineStr">
+        <is>
+          <t>Notaire, administration, légalisation</t>
+        </is>
+      </c>
+      <c r="C49" s="33" t="inlineStr">
+        <is>
+          <t>forfait</t>
+        </is>
+      </c>
+      <c r="D49" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="35" t="n">
         <v>500</v>
       </c>
-      <c r="F46" s="36" t="n">
+      <c r="F49" s="36" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="37" t="inlineStr">
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="37" t="inlineStr">
         <is>
           <t>Réserve pour imprévus opérationnels</t>
         </is>
       </c>
-      <c r="B47" s="38" t="inlineStr">
+      <c r="B50" s="38" t="inlineStr">
         <is>
           <t>Ajustements terrain non anticipés</t>
         </is>
       </c>
-      <c r="C47" s="39" t="inlineStr">
+      <c r="C50" s="39" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D47" s="40" t="n">
+      <c r="D50" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E47" s="41" t="n">
+      <c r="E50" s="41" t="n">
         <v>500</v>
       </c>
-      <c r="F47" s="42" t="n">
+      <c r="F50" s="42" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="43" t="inlineStr">
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="43" t="inlineStr">
         <is>
           <t>Sous-total Autres coûts directs</t>
         </is>
       </c>
-      <c r="E48" s="44" t="n">
+      <c r="E51" s="44" t="n">
         <v>1000</v>
       </c>
-      <c r="F48" s="17" t="inlineStr">
-        <is>
-          <t>0.4%</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="24" customHeight="1">
-      <c r="A49" s="45" t="inlineStr">
+      <c r="F51" s="17" t="inlineStr">
+        <is>
+          <t>0.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="24" customHeight="1">
+      <c r="A52" s="45" t="inlineStr">
         <is>
           <t>TOTAL DES COÛTS DIRECTS</t>
         </is>
       </c>
-      <c r="E49" s="46" t="n">
-        <v>238083</v>
-      </c>
-      <c r="F49" s="47" t="inlineStr">
+      <c r="E52" s="46" t="n">
+        <v>220167</v>
+      </c>
+      <c r="F52" s="47" t="inlineStr">
         <is>
           <t>100 %</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="43" t="inlineStr">
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="43" t="inlineStr">
         <is>
           <t>Frais généraux / Coûts indirects (5 % des coûts directs)</t>
         </is>
       </c>
-      <c r="E50" s="44" t="n">
-        <v>11904</v>
-      </c>
-      <c r="F50" s="48" t="inlineStr">
-        <is>
-          <t>5 % × 238 083</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="28" customHeight="1">
-      <c r="A51" s="18" t="inlineStr">
+      <c r="E53" s="44" t="n">
+        <v>11008</v>
+      </c>
+      <c r="F53" s="48" t="inlineStr">
+        <is>
+          <t>5 % × 220 167</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="28" customHeight="1">
+      <c r="A54" s="18" t="inlineStr">
         <is>
           <t>GRAND TOTAL — BUDGET CASH DEMANDÉ  (plafond Cat. 3 : 250 000 USD)</t>
         </is>
       </c>
-      <c r="E51" s="49" t="n">
-        <v>249987</v>
-      </c>
-      <c r="F51" s="50" t="inlineStr">
+      <c r="E54" s="49" t="n">
+        <v>231175</v>
+      </c>
+      <c r="F54" s="50" t="inlineStr">
         <is>
           <t>&lt; 250 000 USD ✓</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="51" t="inlineStr">
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="51" t="inlineStr">
         <is>
           <t>9. RESSOURCES DE CALCUL GCP — Q18  (crédits séparés du budget cash — plafond 400 000 USD)</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="22" customHeight="1">
-      <c r="A54" s="31" t="inlineStr">
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="31" t="inlineStr">
         <is>
           <t>Vertex AI Custom Training — fine-tuning NLLB LoRA (6 langues × 18 dialectes)</t>
         </is>
       </c>
-      <c r="B54" s="32" t="inlineStr">
+      <c r="B57" s="32" t="inlineStr">
         <is>
           <t>L4 Spot ~0,28 $/h — expérimentations + runs finaux</t>
         </is>
       </c>
-      <c r="C54" s="33" t="inlineStr">
+      <c r="C57" s="33" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D54" s="34" t="n">
+      <c r="D57" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="E54" s="35" t="n">
+      <c r="E57" s="35" t="n">
         <v>45000</v>
       </c>
-      <c r="F54" s="36" t="n">
+      <c r="F57" s="36" t="n">
         <v>45000</v>
       </c>
     </row>
-    <row r="55" ht="22" customHeight="1">
-      <c r="A55" s="37" t="inlineStr">
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="37" t="inlineStr">
         <is>
           <t>Vertex AI Custom Training — fine-tuning MMS-TTS VITS (18 dialectes)</t>
         </is>
       </c>
-      <c r="B55" s="38" t="inlineStr">
+      <c r="B58" s="38" t="inlineStr">
         <is>
           <t>18 dialectes × 3 cycles × 1,5 h GPU + hyperparamètres</t>
         </is>
       </c>
-      <c r="C55" s="39" t="inlineStr">
+      <c r="C58" s="39" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D55" s="40" t="n">
+      <c r="D58" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E55" s="41" t="n">
+      <c r="E58" s="41" t="n">
         <v>20000</v>
       </c>
-      <c r="F55" s="42" t="n">
+      <c r="F58" s="42" t="n">
         <v>20000</v>
       </c>
     </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="31" t="inlineStr">
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="31" t="inlineStr">
         <is>
           <t>Vertex AI Custom Training — buffer expérimentation &amp; réentraînement</t>
         </is>
       </c>
-      <c r="B56" s="32" t="inlineStr">
+      <c r="B59" s="32" t="inlineStr">
         <is>
           <t>Nouvelles données M10–M18, réentraînements itératifs</t>
         </is>
       </c>
-      <c r="C56" s="33" t="inlineStr">
+      <c r="C59" s="33" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D56" s="34" t="n">
+      <c r="D59" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="E56" s="35" t="n">
+      <c r="E59" s="35" t="n">
         <v>15000</v>
       </c>
-      <c r="F56" s="36" t="n">
+      <c r="F59" s="36" t="n">
         <v>15000</v>
       </c>
     </row>
-    <row r="57" ht="22" customHeight="1">
-      <c r="A57" s="37" t="inlineStr">
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="37" t="inlineStr">
         <is>
           <t>Cloud Run GPU (NVIDIA L4 24 Go) — API MGVaovao en production</t>
         </is>
       </c>
-      <c r="B57" s="38" t="inlineStr">
+      <c r="B60" s="38" t="inlineStr">
         <is>
           <t>~2 500 $/mois × 18 mois — scale-to-zero hors heures</t>
         </is>
       </c>
-      <c r="C57" s="39" t="inlineStr">
+      <c r="C60" s="39" t="inlineStr">
         <is>
           <t>mois</t>
         </is>
       </c>
-      <c r="D57" s="40" t="n">
+      <c r="D60" s="40" t="n">
         <v>18</v>
       </c>
-      <c r="E57" s="41" t="n">
+      <c r="E60" s="41" t="n">
         <v>2500</v>
       </c>
-      <c r="F57" s="42" t="n">
+      <c r="F60" s="42" t="n">
         <v>45000</v>
       </c>
     </row>
-    <row r="58" ht="22" customHeight="1">
-      <c r="A58" s="31" t="inlineStr">
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="31" t="inlineStr">
         <is>
           <t>GCS — stockage corpus audio + checkpoints (≈ 3 To)</t>
         </is>
       </c>
-      <c r="B58" s="32" t="inlineStr">
+      <c r="B61" s="32" t="inlineStr">
         <is>
           <t>0,02 $/Go/mois × 3 000 Go × 18 mois + egress</t>
         </is>
       </c>
-      <c r="C58" s="33" t="inlineStr">
+      <c r="C61" s="33" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D58" s="34" t="n">
+      <c r="D61" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="E58" s="35" t="n">
+      <c r="E61" s="35" t="n">
         <v>1500</v>
       </c>
-      <c r="F58" s="36" t="n">
+      <c r="F61" s="36" t="n">
         <v>1500</v>
       </c>
     </row>
-    <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="37" t="inlineStr">
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="37" t="inlineStr">
         <is>
           <t>Vertex AI Pipelines — orchestration MLOps Kubeflow DAG</t>
         </is>
       </c>
-      <c r="B59" s="38" t="inlineStr">
+      <c r="B62" s="38" t="inlineStr">
         <is>
           <t>0,03 $/run × ~500 runs + monitoring continu</t>
         </is>
       </c>
-      <c r="C59" s="39" t="inlineStr">
+      <c r="C62" s="39" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D59" s="40" t="n">
+      <c r="D62" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E59" s="41" t="n">
+      <c r="E62" s="41" t="n">
         <v>500</v>
       </c>
-      <c r="F59" s="42" t="n">
+      <c r="F62" s="42" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="60" ht="22" customHeight="1">
-      <c r="A60" s="31" t="inlineStr">
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="31" t="inlineStr">
         <is>
           <t>Cloud Build, Artifact Registry, Cloud Monitoring, Pub/Sub</t>
         </is>
       </c>
-      <c r="B60" s="32" t="inlineStr">
+      <c r="B63" s="32" t="inlineStr">
         <is>
           <t>CI/CD, registre d'images, alertes, déclencheurs GCS</t>
         </is>
       </c>
-      <c r="C60" s="33" t="inlineStr">
+      <c r="C63" s="33" t="inlineStr">
         <is>
           <t>mois</t>
         </is>
       </c>
-      <c r="D60" s="34" t="n">
+      <c r="D63" s="34" t="n">
         <v>18</v>
       </c>
-      <c r="E60" s="35" t="n">
+      <c r="E63" s="35" t="n">
         <v>139</v>
       </c>
-      <c r="F60" s="36" t="n">
+      <c r="F63" s="36" t="n">
         <v>2500</v>
       </c>
     </row>
-    <row r="61" ht="22" customHeight="1">
-      <c r="A61" s="37" t="inlineStr">
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="37" t="inlineStr">
         <is>
           <t>Dataflow / ingestion pipeline audio — traitement et normalisation</t>
         </is>
       </c>
-      <c r="B61" s="38" t="inlineStr">
+      <c r="B64" s="38" t="inlineStr">
         <is>
           <t>Ingestion et prétraitement audio en pipeline GCS</t>
         </is>
       </c>
-      <c r="C61" s="39" t="inlineStr">
+      <c r="C64" s="39" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="D61" s="40" t="n">
+      <c r="D64" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E61" s="41" t="n">
+      <c r="E64" s="41" t="n">
         <v>20500</v>
       </c>
-      <c r="F61" s="42" t="n">
+      <c r="F64" s="42" t="n">
         <v>20500</v>
       </c>
     </row>
-    <row r="62" ht="28" customHeight="1">
-      <c r="A62" s="21" t="inlineStr">
+    <row r="65" ht="28" customHeight="1">
+      <c r="A65" s="21" t="inlineStr">
         <is>
           <t>TOTAL CRÉDITS GCP DEMANDÉS  (Q18b — séparé du budget cash)</t>
         </is>
       </c>
-      <c r="E62" s="52" t="n">
+      <c r="E65" s="52" t="n">
         <v>150000</v>
       </c>
-      <c r="F62" s="53" t="inlineStr">
+      <c r="F65" s="53" t="inlineStr">
         <is>
           <t>&lt; 400 000 USD ✓</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="23">
-    <mergeCell ref="A41:F41"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A44:D44"/>
+  <mergeCells count="21">
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A56:F56"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="A48:D48"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A24:D24"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A49:D49"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="A43:F43"/>
     <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="A65:D65"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A24:F24"/>
     <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="A50:D50"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A45:F45"/>
-    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A42:D42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2498,7 +2604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2550,16 +2656,16 @@
         </is>
       </c>
       <c r="B4" s="58" t="n">
-        <v>192852</v>
+        <v>152436</v>
       </c>
       <c r="C4" s="59" t="inlineStr">
         <is>
-          <t>81.0 %</t>
+          <t>69.2 %</t>
         </is>
       </c>
       <c r="D4" s="59" t="inlineStr">
         <is>
-          <t>13 postes : 5 direction + 8 développeurs à 1 500 000 MGA/mois — 18 mois</t>
+          <t>12 postes : 5 direction + 7 développeurs à 1 500 000 MGA/mois — 18 mois</t>
         </is>
       </c>
     </row>
@@ -2574,7 +2680,7 @@
       </c>
       <c r="C5" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 3.4 %</t>
+          <t xml:space="preserve"> 3.6 %</t>
         </is>
       </c>
       <c r="D5" s="62" t="inlineStr">
@@ -2586,265 +2692,245 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="57" t="inlineStr">
         <is>
-          <t>3. Collecte terrain</t>
+          <t>3. Collecte et traitement des données</t>
         </is>
       </c>
       <c r="B6" s="58" t="n">
-        <v>10640</v>
+        <v>14231</v>
       </c>
       <c r="C6" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 4.5 %</t>
+          <t xml:space="preserve"> 6.5 %</t>
         </is>
       </c>
       <c r="D6" s="59" t="inlineStr">
         <is>
-          <t>20 collecteurs × 133 USD/mois × 4 mois</t>
+          <t>20 collecteurs × 133 USD × 4 mois + 9 annotateurs × 133 USD × 3 mois</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="60" t="inlineStr">
         <is>
-          <t>4. Annotation et ground truth</t>
+          <t>4. Déplacements et terrain</t>
         </is>
       </c>
       <c r="B7" s="61" t="n">
-        <v>3591</v>
+        <v>20000</v>
       </c>
       <c r="C7" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 1.5 %</t>
+          <t xml:space="preserve"> 9.1 %</t>
         </is>
       </c>
       <c r="D7" s="62" t="inlineStr">
         <is>
-          <t>9 annotateurs × 133 USD/mois × 3 mois</t>
+          <t>14 régions × 2 missions + transport coordinateurs + salles</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="57" t="inlineStr">
         <is>
-          <t>5. Déplacements et terrain</t>
+          <t>5. Formation et ateliers</t>
         </is>
       </c>
       <c r="B8" s="58" t="n">
-        <v>16000</v>
+        <v>22000</v>
       </c>
       <c r="C8" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 6.7 %</t>
+          <t>10.0 %</t>
         </is>
       </c>
       <c r="D8" s="59" t="inlineStr">
         <is>
-          <t>18 régions × 2 missions — avion, per diem, salles</t>
+          <t>Tournée nationale 18 villes + coordinateurs + restitution + IndabaX</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="60" t="inlineStr">
         <is>
-          <t>6. Formation et ateliers</t>
+          <t>6. Communication et mobilisation</t>
         </is>
       </c>
       <c r="B9" s="61" t="n">
-        <v>4500</v>
+        <v>2500</v>
       </c>
       <c r="C9" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 1.9 %</t>
+          <t xml:space="preserve"> 1.1 %</t>
         </is>
       </c>
       <c r="D9" s="62" t="inlineStr">
         <is>
-          <t>Formation équipes terrain + atelier restitution + conférence</t>
+          <t>Rapports semestriels, outils numériques, stratégie réseaux sociaux</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="57" t="inlineStr">
         <is>
-          <t>7. Communication et documentation</t>
+          <t>7. Autres coûts directs</t>
         </is>
       </c>
       <c r="B10" s="58" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="C10" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 0.6 %</t>
+          <t xml:space="preserve"> 0.5 %</t>
         </is>
       </c>
       <c r="D10" s="59" t="inlineStr">
         <is>
-          <t>Rapports semestriels, outils numériques</t>
+          <t>Frais administratifs + réserve imprévus</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="60" t="inlineStr">
-        <is>
-          <t>8. Autres coûts directs</t>
-        </is>
-      </c>
-      <c r="B11" s="61" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C11" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 0.4 %</t>
-        </is>
-      </c>
-      <c r="D11" s="62" t="inlineStr">
-        <is>
-          <t>Frais administratifs + réserve imprévus</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="63" t="inlineStr">
+      <c r="A11" s="63" t="inlineStr">
         <is>
           <t>TOTAL DES COÛTS DIRECTS</t>
         </is>
       </c>
-      <c r="B12" s="46" t="n">
-        <v>238083</v>
-      </c>
-      <c r="C12" s="47" t="inlineStr">
+      <c r="B11" s="46" t="n">
+        <v>220167</v>
+      </c>
+      <c r="C11" s="47" t="inlineStr">
         <is>
           <t>100 %</t>
         </is>
       </c>
-      <c r="D12" s="47" t="inlineStr">
-        <is>
-          <t>238 083 USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="64" t="inlineStr">
+      <c r="D11" s="47" t="inlineStr">
+        <is>
+          <t>220 167 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="64" t="inlineStr">
         <is>
           <t>Frais généraux / indirects (5 %)</t>
         </is>
       </c>
-      <c r="B13" s="44" t="n">
-        <v>11904</v>
-      </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="B12" s="44" t="n">
+        <v>11008</v>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>5 %</t>
         </is>
       </c>
-      <c r="D13" s="17" t="inlineStr">
-        <is>
-          <t>5 % × 238 083</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="65" t="inlineStr">
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>5 % × 220 167</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="65" t="inlineStr">
         <is>
           <t>GRAND TOTAL — BUDGET CASH DEMANDÉ</t>
         </is>
       </c>
-      <c r="B14" s="49" t="n">
-        <v>249987</v>
-      </c>
-      <c r="C14" s="66" t="inlineStr">
+      <c r="B13" s="49" t="n">
+        <v>231175</v>
+      </c>
+      <c r="C13" s="66" t="inlineStr">
         <is>
           <t>&lt; 250 000 USD ✓</t>
         </is>
       </c>
-      <c r="D14" s="66" t="inlineStr">
+      <c r="D13" s="66" t="inlineStr">
         <is>
           <t>Plafond Cat. 3 respecté</t>
         </is>
       </c>
     </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="67" t="inlineStr">
+        <is>
+          <t>RESSOURCES DE CALCUL GCP — Q18  (séparées du budget cash — plafond 400 000 USD)</t>
+        </is>
+      </c>
+    </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="67" t="inlineStr">
-        <is>
-          <t>RESSOURCES DE CALCUL GCP — Q18  (séparées du budget cash — plafond 400 000 USD)</t>
+      <c r="A16" s="57" t="inlineStr">
+        <is>
+          <t>Vertex AI Custom Training — NLLB LoRA + MMS-TTS + expérimentation</t>
+        </is>
+      </c>
+      <c r="B16" s="58" t="n">
+        <v>80000</v>
+      </c>
+      <c r="C16" s="59" t="inlineStr">
+        <is>
+          <t>53.3 %</t>
+        </is>
+      </c>
+      <c r="D16" s="59" t="inlineStr">
+        <is>
+          <t>6 langues × 18 dialectes + cycles itératifs</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="57" t="inlineStr">
-        <is>
-          <t>Vertex AI Custom Training — NLLB LoRA + MMS-TTS + expérimentation</t>
-        </is>
-      </c>
-      <c r="B17" s="58" t="n">
-        <v>80000</v>
-      </c>
-      <c r="C17" s="59" t="inlineStr">
-        <is>
-          <t>53.3 %</t>
-        </is>
-      </c>
-      <c r="D17" s="59" t="inlineStr">
-        <is>
-          <t>6 langues × 18 dialectes + cycles itératifs</t>
+      <c r="A17" s="60" t="inlineStr">
+        <is>
+          <t>Cloud Run GPU — infrastructure de production API (18 mois)</t>
+        </is>
+      </c>
+      <c r="B17" s="61" t="n">
+        <v>45000</v>
+      </c>
+      <c r="C17" s="62" t="inlineStr">
+        <is>
+          <t>30.0 %</t>
+        </is>
+      </c>
+      <c r="D17" s="62" t="inlineStr">
+        <is>
+          <t>NVIDIA L4 24 Go — scale-to-zero hors heures</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="60" t="inlineStr">
-        <is>
-          <t>Cloud Run GPU — infrastructure de production API (18 mois)</t>
-        </is>
-      </c>
-      <c r="B18" s="61" t="n">
-        <v>45000</v>
-      </c>
-      <c r="C18" s="62" t="inlineStr">
-        <is>
-          <t>30.0 %</t>
-        </is>
-      </c>
-      <c r="D18" s="62" t="inlineStr">
-        <is>
-          <t>NVIDIA L4 24 Go — scale-to-zero hors heures</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="57" t="inlineStr">
+      <c r="A18" s="57" t="inlineStr">
         <is>
           <t>GCS, Pipelines, CI/CD, Monitoring, Dataflow, Pub/Sub</t>
         </is>
       </c>
-      <c r="B19" s="58" t="n">
+      <c r="B18" s="58" t="n">
         <v>25000</v>
       </c>
-      <c r="C19" s="59" t="inlineStr">
+      <c r="C18" s="59" t="inlineStr">
         <is>
           <t>16.7 %</t>
         </is>
       </c>
-      <c r="D19" s="59" t="inlineStr">
+      <c r="D18" s="59" t="inlineStr">
         <is>
           <t>Stockage 3 To + orchestration MLOps + ingestion</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="68" t="inlineStr">
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="68" t="inlineStr">
         <is>
           <t>TOTAL CRÉDITS GCP DEMANDÉS (Q18b)</t>
         </is>
       </c>
-      <c r="B20" s="52" t="n">
+      <c r="B19" s="52" t="n">
         <v>150000</v>
       </c>
-      <c r="C20" s="69" t="inlineStr">
+      <c r="C19" s="69" t="inlineStr">
         <is>
           <t>&lt; 400 000 USD ✓</t>
         </is>
       </c>
-      <c r="D20" s="69" t="inlineStr">
+      <c r="D19" s="69" t="inlineStr">
         <is>
           <t>Plafond Q18 respecté</t>
         </is>
@@ -2853,8 +2939,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A16:D16"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A15:D15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>